<commit_message>
Forecast P&L: add technical support hires, founder-led sales
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016qBnaLCMscxuNh2PpcPX2U
</commit_message>
<xml_diff>
--- a/docs/OnSite-forecast-PnL.xlsx
+++ b/docs/OnSite-forecast-PnL.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="106">
   <si>
     <t xml:space="preserve">OnSite - forecast assumptions (blue = editable inputs). All amounts AUD, excluding GST.</t>
   </si>
@@ -95,10 +95,10 @@
     <t xml:space="preserve">A$3/month each (docs/TWILIO.md)</t>
   </si>
   <si>
-    <t xml:space="preserve">Customer support</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ASSUMED ~0.5 hr/park/month</t>
+    <t xml:space="preserve">Support tools &amp; helpdesk software (per park)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASSUMED; support labour is now the hires below</t>
   </si>
   <si>
     <t xml:space="preserve">Hosting variable (per park)</t>
@@ -107,16 +107,28 @@
     <t xml:space="preserve">ONE-OFF / FIXED</t>
   </si>
   <si>
-    <t xml:space="preserve">Sales &amp; onboarding cost per new park (CAC)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ASSUMED demos, events, outreach</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Onboarding/setup cost per new park</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ASSUMED NewBook link, number setup</t>
+    <t xml:space="preserve">Sales cost per new park (non-labour)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASSUMED travel, events, demo costs; founder does the selling (in salary)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Onboarding cost per new park (non-labour)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASSUMED test calls/SMS; labour is the tech support hire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Technical support hire: monthly cost (fully loaded)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASSUMED ~A$80k salary + super and on-costs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First hire starts in month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Second hire when parks at start of month reach</t>
   </si>
   <si>
     <t xml:space="preserve">Hosting base (always-on container, DB, logs)</t>
@@ -290,7 +302,16 @@
     <t xml:space="preserve">OPERATING EXPENSES</t>
   </si>
   <si>
-    <t xml:space="preserve">Sales &amp; onboarding</t>
+    <t xml:space="preserve">Sales &amp; onboarding (non-labour)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Support tools &amp; helpdesk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Technical support staff (count)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Technical support salaries</t>
   </si>
   <si>
     <t xml:space="preserve">Hosting base</t>
@@ -704,7 +725,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Y32"/>
+  <dimension ref="A1:Y35"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
@@ -846,7 +867,7 @@
         <v>24</v>
       </c>
       <c r="B16" s="3" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>25</v>
@@ -873,7 +894,7 @@
         <v>28</v>
       </c>
       <c r="B19" s="3" t="n">
-        <v>300</v>
+        <v>150</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>29</v>
@@ -884,7 +905,7 @@
         <v>30</v>
       </c>
       <c r="B20" s="3" t="n">
-        <v>150</v>
+        <v>50</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>31</v>
@@ -895,18 +916,18 @@
         <v>32</v>
       </c>
       <c r="B21" s="3" t="n">
-        <v>150</v>
+        <v>9000</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B22" s="3" t="n">
-        <v>500</v>
+        <v>9</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>20</v>
@@ -914,10 +935,10 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B23" s="3" t="n">
-        <v>1200</v>
+        <v>400</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>20</v>
@@ -925,13 +946,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B24" s="3" t="n">
-        <v>7500</v>
+        <v>150</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -939,254 +960,287 @@
         <v>37</v>
       </c>
       <c r="B25" s="3" t="n">
-        <v>0.25</v>
+        <v>500</v>
       </c>
       <c r="C25" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="0" t="s">
         <v>38</v>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
         <v>39</v>
       </c>
-      <c r="B27" s="0" t="n">
+      <c r="B27" s="3" t="n">
+        <v>7500</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="B30" s="0" t="n">
         <f aca="false">$B$6*$B$7</f>
         <v>65</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="B30" s="0" t="n">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="B33" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="C30" s="0" t="n">
+      <c r="C33" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="D30" s="0" t="n">
+      <c r="D33" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="E30" s="0" t="n">
+      <c r="E33" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="F30" s="0" t="n">
+      <c r="F33" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="G30" s="0" t="n">
+      <c r="G33" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="H30" s="0" t="n">
+      <c r="H33" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="I30" s="0" t="n">
+      <c r="I33" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="J30" s="0" t="n">
+      <c r="J33" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="K30" s="0" t="n">
+      <c r="K33" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="L30" s="0" t="n">
+      <c r="L33" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="M30" s="0" t="n">
+      <c r="M33" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="N30" s="0" t="n">
+      <c r="N33" s="0" t="n">
         <v>13</v>
       </c>
-      <c r="O30" s="0" t="n">
+      <c r="O33" s="0" t="n">
         <v>14</v>
       </c>
-      <c r="P30" s="0" t="n">
+      <c r="P33" s="0" t="n">
         <v>15</v>
       </c>
-      <c r="Q30" s="0" t="n">
+      <c r="Q33" s="0" t="n">
         <v>16</v>
       </c>
-      <c r="R30" s="0" t="n">
+      <c r="R33" s="0" t="n">
         <v>17</v>
       </c>
-      <c r="S30" s="0" t="n">
+      <c r="S33" s="0" t="n">
         <v>18</v>
       </c>
-      <c r="T30" s="0" t="n">
+      <c r="T33" s="0" t="n">
         <v>19</v>
       </c>
-      <c r="U30" s="0" t="n">
+      <c r="U33" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="V30" s="0" t="n">
+      <c r="V33" s="0" t="n">
         <v>21</v>
       </c>
-      <c r="W30" s="0" t="n">
+      <c r="W33" s="0" t="n">
         <v>22</v>
       </c>
-      <c r="X30" s="0" t="n">
+      <c r="X33" s="0" t="n">
         <v>23</v>
       </c>
-      <c r="Y30" s="0" t="n">
+      <c r="Y33" s="0" t="n">
         <v>24</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C34" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D34" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E34" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F34" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G34" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H34" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="I34" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="J34" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="K34" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="L34" s="3" t="n">
         <v>42</v>
       </c>
-      <c r="B31" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C31" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D31" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E31" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F31" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="G31" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="H31" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="I31" s="3" t="n">
-        <v>18</v>
-      </c>
-      <c r="J31" s="3" t="n">
-        <v>26</v>
-      </c>
-      <c r="K31" s="3" t="n">
-        <v>34</v>
-      </c>
-      <c r="L31" s="3" t="n">
-        <v>42</v>
-      </c>
-      <c r="M31" s="3" t="n">
+      <c r="M34" s="3" t="n">
         <v>56</v>
       </c>
-      <c r="N31" s="3" t="n">
+      <c r="N34" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="O31" s="3" t="n">
+      <c r="O34" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="P31" s="3" t="n">
+      <c r="P34" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="Q31" s="3" t="n">
+      <c r="Q34" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="R31" s="3" t="n">
+      <c r="R34" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="S31" s="3" t="n">
+      <c r="S34" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="T31" s="3" t="n">
+      <c r="T34" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="U31" s="3" t="n">
+      <c r="U34" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="V31" s="3" t="n">
+      <c r="V34" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="W31" s="3" t="n">
+      <c r="W34" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="X31" s="3" t="n">
+      <c r="X34" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="Y31" s="3" t="n">
+      <c r="Y34" s="3" t="n">
         <v>30</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="s">
-        <v>43</v>
-      </c>
-      <c r="B32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N32" s="5" t="n">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N35" s="5" t="n">
         <v>0.01</v>
       </c>
-      <c r="O32" s="5" t="n">
+      <c r="O35" s="5" t="n">
         <v>0.01</v>
       </c>
-      <c r="P32" s="5" t="n">
+      <c r="P35" s="5" t="n">
         <v>0.01</v>
       </c>
-      <c r="Q32" s="5" t="n">
+      <c r="Q35" s="5" t="n">
         <v>0.01</v>
       </c>
-      <c r="R32" s="5" t="n">
+      <c r="R35" s="5" t="n">
         <v>0.01</v>
       </c>
-      <c r="S32" s="5" t="n">
+      <c r="S35" s="5" t="n">
         <v>0.01</v>
       </c>
-      <c r="T32" s="5" t="n">
+      <c r="T35" s="5" t="n">
         <v>0.01</v>
       </c>
-      <c r="U32" s="5" t="n">
+      <c r="U35" s="5" t="n">
         <v>0.01</v>
       </c>
-      <c r="V32" s="5" t="n">
+      <c r="V35" s="5" t="n">
         <v>0.01</v>
       </c>
-      <c r="W32" s="5" t="n">
+      <c r="W35" s="5" t="n">
         <v>0.01</v>
       </c>
-      <c r="X32" s="5" t="n">
+      <c r="X35" s="5" t="n">
         <v>0.01</v>
       </c>
-      <c r="Y32" s="5" t="n">
+      <c r="Y35" s="5" t="n">
         <v>0.01</v>
       </c>
     </row>
@@ -1206,7 +1260,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AA31"/>
+  <dimension ref="A1:AA33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -1215,190 +1269,190 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="R2" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="T2" s="2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="U2" s="2" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="V2" s="2" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="W2" s="2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="X2" s="2" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="Y2" s="2" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="Z2" s="2" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="AA2" s="2" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B3" s="6" t="n">
-        <f aca="false">Assumptions!B31</f>
+        <f aca="false">Assumptions!B34</f>
         <v>2</v>
       </c>
       <c r="C3" s="6" t="n">
-        <f aca="false">Assumptions!C31</f>
+        <f aca="false">Assumptions!C34</f>
         <v>2</v>
       </c>
       <c r="D3" s="6" t="n">
-        <f aca="false">Assumptions!D31</f>
+        <f aca="false">Assumptions!D34</f>
         <v>2</v>
       </c>
       <c r="E3" s="6" t="n">
-        <f aca="false">Assumptions!E31</f>
+        <f aca="false">Assumptions!E34</f>
         <v>2</v>
       </c>
       <c r="F3" s="6" t="n">
-        <f aca="false">Assumptions!F31</f>
+        <f aca="false">Assumptions!F34</f>
         <v>2</v>
       </c>
       <c r="G3" s="6" t="n">
-        <f aca="false">Assumptions!G31</f>
+        <f aca="false">Assumptions!G34</f>
         <v>2</v>
       </c>
       <c r="H3" s="6" t="n">
-        <f aca="false">Assumptions!H31</f>
+        <f aca="false">Assumptions!H34</f>
         <v>12</v>
       </c>
       <c r="I3" s="6" t="n">
-        <f aca="false">Assumptions!I31</f>
+        <f aca="false">Assumptions!I34</f>
         <v>18</v>
       </c>
       <c r="J3" s="6" t="n">
-        <f aca="false">Assumptions!J31</f>
+        <f aca="false">Assumptions!J34</f>
         <v>26</v>
       </c>
       <c r="K3" s="6" t="n">
-        <f aca="false">Assumptions!K31</f>
+        <f aca="false">Assumptions!K34</f>
         <v>34</v>
       </c>
       <c r="L3" s="6" t="n">
-        <f aca="false">Assumptions!L31</f>
+        <f aca="false">Assumptions!L34</f>
         <v>42</v>
       </c>
       <c r="M3" s="6" t="n">
-        <f aca="false">Assumptions!M31</f>
+        <f aca="false">Assumptions!M34</f>
         <v>56</v>
       </c>
       <c r="N3" s="6" t="n">
-        <f aca="false">Assumptions!N31</f>
+        <f aca="false">Assumptions!N34</f>
         <v>30</v>
       </c>
       <c r="O3" s="6" t="n">
-        <f aca="false">Assumptions!O31</f>
+        <f aca="false">Assumptions!O34</f>
         <v>30</v>
       </c>
       <c r="P3" s="6" t="n">
-        <f aca="false">Assumptions!P31</f>
+        <f aca="false">Assumptions!P34</f>
         <v>30</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <f aca="false">Assumptions!Q31</f>
+        <f aca="false">Assumptions!Q34</f>
         <v>30</v>
       </c>
       <c r="R3" s="6" t="n">
-        <f aca="false">Assumptions!R31</f>
+        <f aca="false">Assumptions!R34</f>
         <v>30</v>
       </c>
       <c r="S3" s="6" t="n">
-        <f aca="false">Assumptions!S31</f>
+        <f aca="false">Assumptions!S34</f>
         <v>30</v>
       </c>
       <c r="T3" s="6" t="n">
-        <f aca="false">Assumptions!T31</f>
+        <f aca="false">Assumptions!T34</f>
         <v>30</v>
       </c>
       <c r="U3" s="6" t="n">
-        <f aca="false">Assumptions!U31</f>
+        <f aca="false">Assumptions!U34</f>
         <v>30</v>
       </c>
       <c r="V3" s="6" t="n">
-        <f aca="false">Assumptions!V31</f>
+        <f aca="false">Assumptions!V34</f>
         <v>30</v>
       </c>
       <c r="W3" s="6" t="n">
-        <f aca="false">Assumptions!W31</f>
+        <f aca="false">Assumptions!W34</f>
         <v>30</v>
       </c>
       <c r="X3" s="6" t="n">
-        <f aca="false">Assumptions!X31</f>
+        <f aca="false">Assumptions!X34</f>
         <v>30</v>
       </c>
       <c r="Y3" s="6" t="n">
-        <f aca="false">Assumptions!Y31</f>
+        <f aca="false">Assumptions!Y34</f>
         <v>30</v>
       </c>
       <c r="Z3" s="6" t="n">
@@ -1412,102 +1466,102 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B4" s="6" t="n">
-        <f aca="false">B5*Assumptions!B32</f>
+        <f aca="false">B5*Assumptions!B35</f>
         <v>0</v>
       </c>
       <c r="C4" s="6" t="n">
-        <f aca="false">C5*Assumptions!C32</f>
+        <f aca="false">C5*Assumptions!C35</f>
         <v>0</v>
       </c>
       <c r="D4" s="6" t="n">
-        <f aca="false">D5*Assumptions!D32</f>
+        <f aca="false">D5*Assumptions!D35</f>
         <v>0</v>
       </c>
       <c r="E4" s="6" t="n">
-        <f aca="false">E5*Assumptions!E32</f>
+        <f aca="false">E5*Assumptions!E35</f>
         <v>0</v>
       </c>
       <c r="F4" s="6" t="n">
-        <f aca="false">F5*Assumptions!F32</f>
+        <f aca="false">F5*Assumptions!F35</f>
         <v>0</v>
       </c>
       <c r="G4" s="6" t="n">
-        <f aca="false">G5*Assumptions!G32</f>
+        <f aca="false">G5*Assumptions!G35</f>
         <v>0</v>
       </c>
       <c r="H4" s="6" t="n">
-        <f aca="false">H5*Assumptions!H32</f>
+        <f aca="false">H5*Assumptions!H35</f>
         <v>0</v>
       </c>
       <c r="I4" s="6" t="n">
-        <f aca="false">I5*Assumptions!I32</f>
+        <f aca="false">I5*Assumptions!I35</f>
         <v>0</v>
       </c>
       <c r="J4" s="6" t="n">
-        <f aca="false">J5*Assumptions!J32</f>
+        <f aca="false">J5*Assumptions!J35</f>
         <v>0</v>
       </c>
       <c r="K4" s="6" t="n">
-        <f aca="false">K5*Assumptions!K32</f>
+        <f aca="false">K5*Assumptions!K35</f>
         <v>0</v>
       </c>
       <c r="L4" s="6" t="n">
-        <f aca="false">L5*Assumptions!L32</f>
+        <f aca="false">L5*Assumptions!L35</f>
         <v>0</v>
       </c>
       <c r="M4" s="6" t="n">
-        <f aca="false">M5*Assumptions!M32</f>
+        <f aca="false">M5*Assumptions!M35</f>
         <v>0</v>
       </c>
       <c r="N4" s="6" t="n">
-        <f aca="false">N5*Assumptions!N32</f>
+        <f aca="false">N5*Assumptions!N35</f>
         <v>2</v>
       </c>
       <c r="O4" s="6" t="n">
-        <f aca="false">O5*Assumptions!O32</f>
+        <f aca="false">O5*Assumptions!O35</f>
         <v>2.28</v>
       </c>
       <c r="P4" s="6" t="n">
-        <f aca="false">P5*Assumptions!P32</f>
+        <f aca="false">P5*Assumptions!P35</f>
         <v>2.5572</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <f aca="false">Q5*Assumptions!Q32</f>
+        <f aca="false">Q5*Assumptions!Q35</f>
         <v>2.831628</v>
       </c>
       <c r="R4" s="6" t="n">
-        <f aca="false">R5*Assumptions!R32</f>
+        <f aca="false">R5*Assumptions!R35</f>
         <v>3.10331172</v>
       </c>
       <c r="S4" s="6" t="n">
-        <f aca="false">S5*Assumptions!S32</f>
+        <f aca="false">S5*Assumptions!S35</f>
         <v>3.3722786028</v>
       </c>
       <c r="T4" s="6" t="n">
-        <f aca="false">T5*Assumptions!T32</f>
+        <f aca="false">T5*Assumptions!T35</f>
         <v>3.638555816772</v>
       </c>
       <c r="U4" s="6" t="n">
-        <f aca="false">U5*Assumptions!U32</f>
+        <f aca="false">U5*Assumptions!U35</f>
         <v>3.90217025860428</v>
       </c>
       <c r="V4" s="6" t="n">
-        <f aca="false">V5*Assumptions!V32</f>
+        <f aca="false">V5*Assumptions!V35</f>
         <v>4.16314855601824</v>
       </c>
       <c r="W4" s="6" t="n">
-        <f aca="false">W5*Assumptions!W32</f>
+        <f aca="false">W5*Assumptions!W35</f>
         <v>4.42151707045805</v>
       </c>
       <c r="X4" s="6" t="n">
-        <f aca="false">X5*Assumptions!X32</f>
+        <f aca="false">X5*Assumptions!X35</f>
         <v>4.67730189975347</v>
       </c>
       <c r="Y4" s="6" t="n">
-        <f aca="false">Y5*Assumptions!Y32</f>
+        <f aca="false">Y5*Assumptions!Y35</f>
         <v>4.93052888075594</v>
       </c>
       <c r="Z4" s="6" t="n">
@@ -1521,7 +1575,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B5" s="6" t="n">
         <v>0</v>
@@ -1629,7 +1683,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B6" s="6" t="n">
         <f aca="false">B5+B3-B4</f>
@@ -1738,7 +1792,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B7" s="6" t="n">
         <f aca="false">(B5+B6)/2</f>
@@ -1841,102 +1895,102 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B8" s="6" t="n">
-        <f aca="false">B7*Assumptions!$B$27</f>
+        <f aca="false">B7*Assumptions!$B$30</f>
         <v>65</v>
       </c>
       <c r="C8" s="6" t="n">
-        <f aca="false">C7*Assumptions!$B$27</f>
+        <f aca="false">C7*Assumptions!$B$30</f>
         <v>195</v>
       </c>
       <c r="D8" s="6" t="n">
-        <f aca="false">D7*Assumptions!$B$27</f>
+        <f aca="false">D7*Assumptions!$B$30</f>
         <v>325</v>
       </c>
       <c r="E8" s="6" t="n">
-        <f aca="false">E7*Assumptions!$B$27</f>
+        <f aca="false">E7*Assumptions!$B$30</f>
         <v>455</v>
       </c>
       <c r="F8" s="6" t="n">
-        <f aca="false">F7*Assumptions!$B$27</f>
+        <f aca="false">F7*Assumptions!$B$30</f>
         <v>585</v>
       </c>
       <c r="G8" s="6" t="n">
-        <f aca="false">G7*Assumptions!$B$27</f>
+        <f aca="false">G7*Assumptions!$B$30</f>
         <v>715</v>
       </c>
       <c r="H8" s="6" t="n">
-        <f aca="false">H7*Assumptions!$B$27</f>
+        <f aca="false">H7*Assumptions!$B$30</f>
         <v>1170</v>
       </c>
       <c r="I8" s="6" t="n">
-        <f aca="false">I7*Assumptions!$B$27</f>
+        <f aca="false">I7*Assumptions!$B$30</f>
         <v>2145</v>
       </c>
       <c r="J8" s="6" t="n">
-        <f aca="false">J7*Assumptions!$B$27</f>
+        <f aca="false">J7*Assumptions!$B$30</f>
         <v>3575</v>
       </c>
       <c r="K8" s="6" t="n">
-        <f aca="false">K7*Assumptions!$B$27</f>
+        <f aca="false">K7*Assumptions!$B$30</f>
         <v>5525</v>
       </c>
       <c r="L8" s="6" t="n">
-        <f aca="false">L7*Assumptions!$B$27</f>
+        <f aca="false">L7*Assumptions!$B$30</f>
         <v>7995</v>
       </c>
       <c r="M8" s="6" t="n">
-        <f aca="false">M7*Assumptions!$B$27</f>
+        <f aca="false">M7*Assumptions!$B$30</f>
         <v>11180</v>
       </c>
       <c r="N8" s="6" t="n">
-        <f aca="false">N7*Assumptions!$B$27</f>
+        <f aca="false">N7*Assumptions!$B$30</f>
         <v>13910</v>
       </c>
       <c r="O8" s="6" t="n">
-        <f aca="false">O7*Assumptions!$B$27</f>
+        <f aca="false">O7*Assumptions!$B$30</f>
         <v>15720.9</v>
       </c>
       <c r="P8" s="6" t="n">
-        <f aca="false">P7*Assumptions!$B$27</f>
+        <f aca="false">P7*Assumptions!$B$30</f>
         <v>17513.691</v>
       </c>
       <c r="Q8" s="6" t="n">
-        <f aca="false">Q7*Assumptions!$B$27</f>
+        <f aca="false">Q7*Assumptions!$B$30</f>
         <v>19288.55409</v>
       </c>
       <c r="R8" s="6" t="n">
-        <f aca="false">R7*Assumptions!$B$27</f>
+        <f aca="false">R7*Assumptions!$B$30</f>
         <v>21045.6685491</v>
       </c>
       <c r="S8" s="6" t="n">
-        <f aca="false">S7*Assumptions!$B$27</f>
+        <f aca="false">S7*Assumptions!$B$30</f>
         <v>22785.211863609</v>
       </c>
       <c r="T8" s="6" t="n">
-        <f aca="false">T7*Assumptions!$B$27</f>
+        <f aca="false">T7*Assumptions!$B$30</f>
         <v>24507.3597449729</v>
       </c>
       <c r="U8" s="6" t="n">
-        <f aca="false">U7*Assumptions!$B$27</f>
+        <f aca="false">U7*Assumptions!$B$30</f>
         <v>26212.2861475232</v>
       </c>
       <c r="V8" s="6" t="n">
-        <f aca="false">V7*Assumptions!$B$27</f>
+        <f aca="false">V7*Assumptions!$B$30</f>
         <v>27900.1632860479</v>
       </c>
       <c r="W8" s="6" t="n">
-        <f aca="false">W7*Assumptions!$B$27</f>
+        <f aca="false">W7*Assumptions!$B$30</f>
         <v>29571.1616531875</v>
       </c>
       <c r="X8" s="6" t="n">
-        <f aca="false">X7*Assumptions!$B$27</f>
+        <f aca="false">X7*Assumptions!$B$30</f>
         <v>31225.4500366556</v>
       </c>
       <c r="Y8" s="6" t="n">
-        <f aca="false">Y7*Assumptions!$B$27</f>
+        <f aca="false">Y7*Assumptions!$B$30</f>
         <v>32863.195536289</v>
       </c>
       <c r="Z8" s="6" t="n">
@@ -1950,7 +2004,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
@@ -1981,7 +2035,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B10" s="6" t="n">
         <f aca="false">B7*Assumptions!$B$4</f>
@@ -2090,7 +2144,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B11" s="6" t="n">
         <f aca="false">B8*Assumptions!$B$5</f>
@@ -2199,7 +2253,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B12" s="7" t="n">
         <f aca="false">B10+B11</f>
@@ -2308,7 +2362,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B13" s="6"/>
       <c r="C13" s="6"/>
@@ -2339,7 +2393,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B14" s="6" t="n">
         <f aca="false">B8*(Assumptions!$B$9+Assumptions!$B$10+Assumptions!$B$11+Assumptions!$B$12+Assumptions!$B$13)</f>
@@ -2448,7 +2502,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B15" s="6" t="n">
         <f aca="false">B7*Assumptions!$B$15</f>
@@ -2557,7 +2611,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B16" s="6" t="n">
         <f aca="false">B7*Assumptions!$B$17</f>
@@ -2666,7 +2720,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B17" s="6" t="n">
         <f aca="false">B14+B15+B16</f>
@@ -2775,7 +2829,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B18" s="7" t="n">
         <f aca="false">B12-B17</f>
@@ -2884,7 +2938,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">B18/B12</f>
@@ -2993,7 +3047,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B20" s="6"/>
       <c r="C20" s="6"/>
@@ -3024,1201 +3078,1419 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="B21" s="6" t="n">
         <f aca="false">B3*(Assumptions!$B$19+Assumptions!$B$20)</f>
-        <v>900</v>
+        <v>400</v>
       </c>
       <c r="C21" s="6" t="n">
         <f aca="false">C3*(Assumptions!$B$19+Assumptions!$B$20)</f>
-        <v>900</v>
+        <v>400</v>
       </c>
       <c r="D21" s="6" t="n">
         <f aca="false">D3*(Assumptions!$B$19+Assumptions!$B$20)</f>
-        <v>900</v>
+        <v>400</v>
       </c>
       <c r="E21" s="6" t="n">
         <f aca="false">E3*(Assumptions!$B$19+Assumptions!$B$20)</f>
-        <v>900</v>
+        <v>400</v>
       </c>
       <c r="F21" s="6" t="n">
         <f aca="false">F3*(Assumptions!$B$19+Assumptions!$B$20)</f>
-        <v>900</v>
+        <v>400</v>
       </c>
       <c r="G21" s="6" t="n">
         <f aca="false">G3*(Assumptions!$B$19+Assumptions!$B$20)</f>
-        <v>900</v>
+        <v>400</v>
       </c>
       <c r="H21" s="6" t="n">
         <f aca="false">H3*(Assumptions!$B$19+Assumptions!$B$20)</f>
-        <v>5400</v>
+        <v>2400</v>
       </c>
       <c r="I21" s="6" t="n">
         <f aca="false">I3*(Assumptions!$B$19+Assumptions!$B$20)</f>
-        <v>8100</v>
+        <v>3600</v>
       </c>
       <c r="J21" s="6" t="n">
         <f aca="false">J3*(Assumptions!$B$19+Assumptions!$B$20)</f>
-        <v>11700</v>
+        <v>5200</v>
       </c>
       <c r="K21" s="6" t="n">
         <f aca="false">K3*(Assumptions!$B$19+Assumptions!$B$20)</f>
-        <v>15300</v>
+        <v>6800</v>
       </c>
       <c r="L21" s="6" t="n">
         <f aca="false">L3*(Assumptions!$B$19+Assumptions!$B$20)</f>
-        <v>18900</v>
+        <v>8400</v>
       </c>
       <c r="M21" s="6" t="n">
         <f aca="false">M3*(Assumptions!$B$19+Assumptions!$B$20)</f>
-        <v>25200</v>
+        <v>11200</v>
       </c>
       <c r="N21" s="6" t="n">
         <f aca="false">N3*(Assumptions!$B$19+Assumptions!$B$20)</f>
-        <v>13500</v>
+        <v>6000</v>
       </c>
       <c r="O21" s="6" t="n">
         <f aca="false">O3*(Assumptions!$B$19+Assumptions!$B$20)</f>
-        <v>13500</v>
+        <v>6000</v>
       </c>
       <c r="P21" s="6" t="n">
         <f aca="false">P3*(Assumptions!$B$19+Assumptions!$B$20)</f>
-        <v>13500</v>
+        <v>6000</v>
       </c>
       <c r="Q21" s="6" t="n">
         <f aca="false">Q3*(Assumptions!$B$19+Assumptions!$B$20)</f>
-        <v>13500</v>
+        <v>6000</v>
       </c>
       <c r="R21" s="6" t="n">
         <f aca="false">R3*(Assumptions!$B$19+Assumptions!$B$20)</f>
-        <v>13500</v>
+        <v>6000</v>
       </c>
       <c r="S21" s="6" t="n">
         <f aca="false">S3*(Assumptions!$B$19+Assumptions!$B$20)</f>
-        <v>13500</v>
+        <v>6000</v>
       </c>
       <c r="T21" s="6" t="n">
         <f aca="false">T3*(Assumptions!$B$19+Assumptions!$B$20)</f>
-        <v>13500</v>
+        <v>6000</v>
       </c>
       <c r="U21" s="6" t="n">
         <f aca="false">U3*(Assumptions!$B$19+Assumptions!$B$20)</f>
-        <v>13500</v>
+        <v>6000</v>
       </c>
       <c r="V21" s="6" t="n">
         <f aca="false">V3*(Assumptions!$B$19+Assumptions!$B$20)</f>
-        <v>13500</v>
+        <v>6000</v>
       </c>
       <c r="W21" s="6" t="n">
         <f aca="false">W3*(Assumptions!$B$19+Assumptions!$B$20)</f>
-        <v>13500</v>
+        <v>6000</v>
       </c>
       <c r="X21" s="6" t="n">
         <f aca="false">X3*(Assumptions!$B$19+Assumptions!$B$20)</f>
-        <v>13500</v>
+        <v>6000</v>
       </c>
       <c r="Y21" s="6" t="n">
         <f aca="false">Y3*(Assumptions!$B$19+Assumptions!$B$20)</f>
-        <v>13500</v>
+        <v>6000</v>
       </c>
       <c r="Z21" s="6" t="n">
         <f aca="false">SUM(B21:M21)</f>
-        <v>90000</v>
+        <v>40000</v>
       </c>
       <c r="AA21" s="6" t="n">
         <f aca="false">SUM(N21:Y21)</f>
-        <v>162000</v>
+        <v>72000</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>24</v>
+        <v>94</v>
       </c>
       <c r="B22" s="6" t="n">
         <f aca="false">B7*Assumptions!$B$16</f>
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="C22" s="6" t="n">
         <f aca="false">C7*Assumptions!$B$16</f>
-        <v>75</v>
+        <v>15</v>
       </c>
       <c r="D22" s="6" t="n">
         <f aca="false">D7*Assumptions!$B$16</f>
-        <v>125</v>
+        <v>25</v>
       </c>
       <c r="E22" s="6" t="n">
         <f aca="false">E7*Assumptions!$B$16</f>
-        <v>175</v>
+        <v>35</v>
       </c>
       <c r="F22" s="6" t="n">
         <f aca="false">F7*Assumptions!$B$16</f>
-        <v>225</v>
+        <v>45</v>
       </c>
       <c r="G22" s="6" t="n">
         <f aca="false">G7*Assumptions!$B$16</f>
-        <v>275</v>
+        <v>55</v>
       </c>
       <c r="H22" s="6" t="n">
         <f aca="false">H7*Assumptions!$B$16</f>
-        <v>450</v>
+        <v>90</v>
       </c>
       <c r="I22" s="6" t="n">
         <f aca="false">I7*Assumptions!$B$16</f>
-        <v>825</v>
+        <v>165</v>
       </c>
       <c r="J22" s="6" t="n">
         <f aca="false">J7*Assumptions!$B$16</f>
-        <v>1375</v>
+        <v>275</v>
       </c>
       <c r="K22" s="6" t="n">
         <f aca="false">K7*Assumptions!$B$16</f>
-        <v>2125</v>
+        <v>425</v>
       </c>
       <c r="L22" s="6" t="n">
         <f aca="false">L7*Assumptions!$B$16</f>
-        <v>3075</v>
+        <v>615</v>
       </c>
       <c r="M22" s="6" t="n">
         <f aca="false">M7*Assumptions!$B$16</f>
-        <v>4300</v>
+        <v>860</v>
       </c>
       <c r="N22" s="6" t="n">
         <f aca="false">N7*Assumptions!$B$16</f>
-        <v>5350</v>
+        <v>1070</v>
       </c>
       <c r="O22" s="6" t="n">
         <f aca="false">O7*Assumptions!$B$16</f>
-        <v>6046.5</v>
+        <v>1209.3</v>
       </c>
       <c r="P22" s="6" t="n">
         <f aca="false">P7*Assumptions!$B$16</f>
-        <v>6736.035</v>
+        <v>1347.207</v>
       </c>
       <c r="Q22" s="6" t="n">
         <f aca="false">Q7*Assumptions!$B$16</f>
-        <v>7418.67465</v>
+        <v>1483.73493</v>
       </c>
       <c r="R22" s="6" t="n">
         <f aca="false">R7*Assumptions!$B$16</f>
-        <v>8094.4879035</v>
+        <v>1618.8975807</v>
       </c>
       <c r="S22" s="6" t="n">
         <f aca="false">S7*Assumptions!$B$16</f>
-        <v>8763.543024465</v>
+        <v>1752.708604893</v>
       </c>
       <c r="T22" s="6" t="n">
         <f aca="false">T7*Assumptions!$B$16</f>
-        <v>9425.90759422035</v>
+        <v>1885.18151884407</v>
       </c>
       <c r="U22" s="6" t="n">
         <f aca="false">U7*Assumptions!$B$16</f>
-        <v>10081.6485182781</v>
+        <v>2016.32970365563</v>
       </c>
       <c r="V22" s="6" t="n">
         <f aca="false">V7*Assumptions!$B$16</f>
-        <v>10730.8320330954</v>
+        <v>2146.16640661907</v>
       </c>
       <c r="W22" s="6" t="n">
         <f aca="false">W7*Assumptions!$B$16</f>
-        <v>11373.5237127644</v>
+        <v>2274.70474255288</v>
       </c>
       <c r="X22" s="6" t="n">
         <f aca="false">X7*Assumptions!$B$16</f>
-        <v>12009.7884756368</v>
+        <v>2401.95769512735</v>
       </c>
       <c r="Y22" s="6" t="n">
         <f aca="false">Y7*Assumptions!$B$16</f>
-        <v>12639.6905908804</v>
+        <v>2527.93811817608</v>
       </c>
       <c r="Z22" s="6" t="n">
         <f aca="false">SUM(B22:M22)</f>
-        <v>13050</v>
+        <v>2610</v>
       </c>
       <c r="AA22" s="6" t="n">
         <f aca="false">SUM(N22:Y22)</f>
-        <v>108670.63150284</v>
+        <v>21734.1263005681</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="B23" s="6" t="n">
-        <f aca="false">Assumptions!$B$21</f>
-        <v>150</v>
+        <f aca="false">IF(Assumptions!B33&gt;=Assumptions!$B$22,1,0)+IF(AND(Assumptions!B33&gt;=Assumptions!$B$22,B5&gt;=Assumptions!$B$23),1,0)</f>
+        <v>0</v>
       </c>
       <c r="C23" s="6" t="n">
-        <f aca="false">Assumptions!$B$21</f>
-        <v>150</v>
+        <f aca="false">IF(Assumptions!C33&gt;=Assumptions!$B$22,1,0)+IF(AND(Assumptions!C33&gt;=Assumptions!$B$22,C5&gt;=Assumptions!$B$23),1,0)</f>
+        <v>0</v>
       </c>
       <c r="D23" s="6" t="n">
-        <f aca="false">Assumptions!$B$21</f>
-        <v>150</v>
+        <f aca="false">IF(Assumptions!D33&gt;=Assumptions!$B$22,1,0)+IF(AND(Assumptions!D33&gt;=Assumptions!$B$22,D5&gt;=Assumptions!$B$23),1,0)</f>
+        <v>0</v>
       </c>
       <c r="E23" s="6" t="n">
-        <f aca="false">Assumptions!$B$21</f>
-        <v>150</v>
+        <f aca="false">IF(Assumptions!E33&gt;=Assumptions!$B$22,1,0)+IF(AND(Assumptions!E33&gt;=Assumptions!$B$22,E5&gt;=Assumptions!$B$23),1,0)</f>
+        <v>0</v>
       </c>
       <c r="F23" s="6" t="n">
-        <f aca="false">Assumptions!$B$21</f>
-        <v>150</v>
+        <f aca="false">IF(Assumptions!F33&gt;=Assumptions!$B$22,1,0)+IF(AND(Assumptions!F33&gt;=Assumptions!$B$22,F5&gt;=Assumptions!$B$23),1,0)</f>
+        <v>0</v>
       </c>
       <c r="G23" s="6" t="n">
-        <f aca="false">Assumptions!$B$21</f>
-        <v>150</v>
+        <f aca="false">IF(Assumptions!G33&gt;=Assumptions!$B$22,1,0)+IF(AND(Assumptions!G33&gt;=Assumptions!$B$22,G5&gt;=Assumptions!$B$23),1,0)</f>
+        <v>0</v>
       </c>
       <c r="H23" s="6" t="n">
-        <f aca="false">Assumptions!$B$21</f>
-        <v>150</v>
+        <f aca="false">IF(Assumptions!H33&gt;=Assumptions!$B$22,1,0)+IF(AND(Assumptions!H33&gt;=Assumptions!$B$22,H5&gt;=Assumptions!$B$23),1,0)</f>
+        <v>0</v>
       </c>
       <c r="I23" s="6" t="n">
-        <f aca="false">Assumptions!$B$21</f>
-        <v>150</v>
+        <f aca="false">IF(Assumptions!I33&gt;=Assumptions!$B$22,1,0)+IF(AND(Assumptions!I33&gt;=Assumptions!$B$22,I5&gt;=Assumptions!$B$23),1,0)</f>
+        <v>0</v>
       </c>
       <c r="J23" s="6" t="n">
-        <f aca="false">Assumptions!$B$21</f>
-        <v>150</v>
+        <f aca="false">IF(Assumptions!J33&gt;=Assumptions!$B$22,1,0)+IF(AND(Assumptions!J33&gt;=Assumptions!$B$22,J5&gt;=Assumptions!$B$23),1,0)</f>
+        <v>1</v>
       </c>
       <c r="K23" s="6" t="n">
-        <f aca="false">Assumptions!$B$21</f>
-        <v>150</v>
+        <f aca="false">IF(Assumptions!K33&gt;=Assumptions!$B$22,1,0)+IF(AND(Assumptions!K33&gt;=Assumptions!$B$22,K5&gt;=Assumptions!$B$23),1,0)</f>
+        <v>1</v>
       </c>
       <c r="L23" s="6" t="n">
-        <f aca="false">Assumptions!$B$21</f>
-        <v>150</v>
+        <f aca="false">IF(Assumptions!L33&gt;=Assumptions!$B$22,1,0)+IF(AND(Assumptions!L33&gt;=Assumptions!$B$22,L5&gt;=Assumptions!$B$23),1,0)</f>
+        <v>1</v>
       </c>
       <c r="M23" s="6" t="n">
-        <f aca="false">Assumptions!$B$21</f>
-        <v>150</v>
+        <f aca="false">IF(Assumptions!M33&gt;=Assumptions!$B$22,1,0)+IF(AND(Assumptions!M33&gt;=Assumptions!$B$22,M5&gt;=Assumptions!$B$23),1,0)</f>
+        <v>1</v>
       </c>
       <c r="N23" s="6" t="n">
-        <f aca="false">Assumptions!$B$21</f>
-        <v>150</v>
+        <f aca="false">IF(Assumptions!N33&gt;=Assumptions!$B$22,1,0)+IF(AND(Assumptions!N33&gt;=Assumptions!$B$22,N5&gt;=Assumptions!$B$23),1,0)</f>
+        <v>1</v>
       </c>
       <c r="O23" s="6" t="n">
-        <f aca="false">Assumptions!$B$21</f>
-        <v>150</v>
+        <f aca="false">IF(Assumptions!O33&gt;=Assumptions!$B$22,1,0)+IF(AND(Assumptions!O33&gt;=Assumptions!$B$22,O5&gt;=Assumptions!$B$23),1,0)</f>
+        <v>1</v>
       </c>
       <c r="P23" s="6" t="n">
-        <f aca="false">Assumptions!$B$21</f>
-        <v>150</v>
+        <f aca="false">IF(Assumptions!P33&gt;=Assumptions!$B$22,1,0)+IF(AND(Assumptions!P33&gt;=Assumptions!$B$22,P5&gt;=Assumptions!$B$23),1,0)</f>
+        <v>1</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <f aca="false">Assumptions!$B$21</f>
-        <v>150</v>
+        <f aca="false">IF(Assumptions!Q33&gt;=Assumptions!$B$22,1,0)+IF(AND(Assumptions!Q33&gt;=Assumptions!$B$22,Q5&gt;=Assumptions!$B$23),1,0)</f>
+        <v>1</v>
       </c>
       <c r="R23" s="6" t="n">
-        <f aca="false">Assumptions!$B$21</f>
-        <v>150</v>
+        <f aca="false">IF(Assumptions!R33&gt;=Assumptions!$B$22,1,0)+IF(AND(Assumptions!R33&gt;=Assumptions!$B$22,R5&gt;=Assumptions!$B$23),1,0)</f>
+        <v>1</v>
       </c>
       <c r="S23" s="6" t="n">
-        <f aca="false">Assumptions!$B$21</f>
-        <v>150</v>
+        <f aca="false">IF(Assumptions!S33&gt;=Assumptions!$B$22,1,0)+IF(AND(Assumptions!S33&gt;=Assumptions!$B$22,S5&gt;=Assumptions!$B$23),1,0)</f>
+        <v>1</v>
       </c>
       <c r="T23" s="6" t="n">
-        <f aca="false">Assumptions!$B$21</f>
-        <v>150</v>
+        <f aca="false">IF(Assumptions!T33&gt;=Assumptions!$B$22,1,0)+IF(AND(Assumptions!T33&gt;=Assumptions!$B$22,T5&gt;=Assumptions!$B$23),1,0)</f>
+        <v>1</v>
       </c>
       <c r="U23" s="6" t="n">
-        <f aca="false">Assumptions!$B$21</f>
-        <v>150</v>
+        <f aca="false">IF(Assumptions!U33&gt;=Assumptions!$B$22,1,0)+IF(AND(Assumptions!U33&gt;=Assumptions!$B$22,U5&gt;=Assumptions!$B$23),1,0)</f>
+        <v>1</v>
       </c>
       <c r="V23" s="6" t="n">
-        <f aca="false">Assumptions!$B$21</f>
-        <v>150</v>
+        <f aca="false">IF(Assumptions!V33&gt;=Assumptions!$B$22,1,0)+IF(AND(Assumptions!V33&gt;=Assumptions!$B$22,V5&gt;=Assumptions!$B$23),1,0)</f>
+        <v>2</v>
       </c>
       <c r="W23" s="6" t="n">
-        <f aca="false">Assumptions!$B$21</f>
-        <v>150</v>
+        <f aca="false">IF(Assumptions!W33&gt;=Assumptions!$B$22,1,0)+IF(AND(Assumptions!W33&gt;=Assumptions!$B$22,W5&gt;=Assumptions!$B$23),1,0)</f>
+        <v>2</v>
       </c>
       <c r="X23" s="6" t="n">
-        <f aca="false">Assumptions!$B$21</f>
-        <v>150</v>
+        <f aca="false">IF(Assumptions!X33&gt;=Assumptions!$B$22,1,0)+IF(AND(Assumptions!X33&gt;=Assumptions!$B$22,X5&gt;=Assumptions!$B$23),1,0)</f>
+        <v>2</v>
       </c>
       <c r="Y23" s="6" t="n">
-        <f aca="false">Assumptions!$B$21</f>
-        <v>150</v>
+        <f aca="false">IF(Assumptions!Y33&gt;=Assumptions!$B$22,1,0)+IF(AND(Assumptions!Y33&gt;=Assumptions!$B$22,Y5&gt;=Assumptions!$B$23),1,0)</f>
+        <v>2</v>
       </c>
       <c r="Z23" s="6" t="n">
-        <f aca="false">SUM(B23:M23)</f>
-        <v>1800</v>
+        <f aca="false">M23</f>
+        <v>1</v>
       </c>
       <c r="AA23" s="6" t="n">
-        <f aca="false">SUM(N23:Y23)</f>
-        <v>1800</v>
+        <f aca="false">Y23</f>
+        <v>2</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="B24" s="6" t="n">
-        <f aca="false">Assumptions!$B$22</f>
-        <v>500</v>
+        <f aca="false">B23*Assumptions!$B$21</f>
+        <v>0</v>
       </c>
       <c r="C24" s="6" t="n">
-        <f aca="false">Assumptions!$B$22</f>
-        <v>500</v>
+        <f aca="false">C23*Assumptions!$B$21</f>
+        <v>0</v>
       </c>
       <c r="D24" s="6" t="n">
-        <f aca="false">Assumptions!$B$22</f>
-        <v>500</v>
+        <f aca="false">D23*Assumptions!$B$21</f>
+        <v>0</v>
       </c>
       <c r="E24" s="6" t="n">
-        <f aca="false">Assumptions!$B$22</f>
-        <v>500</v>
+        <f aca="false">E23*Assumptions!$B$21</f>
+        <v>0</v>
       </c>
       <c r="F24" s="6" t="n">
-        <f aca="false">Assumptions!$B$22</f>
-        <v>500</v>
+        <f aca="false">F23*Assumptions!$B$21</f>
+        <v>0</v>
       </c>
       <c r="G24" s="6" t="n">
-        <f aca="false">Assumptions!$B$22</f>
-        <v>500</v>
+        <f aca="false">G23*Assumptions!$B$21</f>
+        <v>0</v>
       </c>
       <c r="H24" s="6" t="n">
-        <f aca="false">Assumptions!$B$22</f>
-        <v>500</v>
+        <f aca="false">H23*Assumptions!$B$21</f>
+        <v>0</v>
       </c>
       <c r="I24" s="6" t="n">
-        <f aca="false">Assumptions!$B$22</f>
-        <v>500</v>
+        <f aca="false">I23*Assumptions!$B$21</f>
+        <v>0</v>
       </c>
       <c r="J24" s="6" t="n">
-        <f aca="false">Assumptions!$B$22</f>
-        <v>500</v>
+        <f aca="false">J23*Assumptions!$B$21</f>
+        <v>9000</v>
       </c>
       <c r="K24" s="6" t="n">
-        <f aca="false">Assumptions!$B$22</f>
-        <v>500</v>
+        <f aca="false">K23*Assumptions!$B$21</f>
+        <v>9000</v>
       </c>
       <c r="L24" s="6" t="n">
-        <f aca="false">Assumptions!$B$22</f>
-        <v>500</v>
+        <f aca="false">L23*Assumptions!$B$21</f>
+        <v>9000</v>
       </c>
       <c r="M24" s="6" t="n">
-        <f aca="false">Assumptions!$B$22</f>
-        <v>500</v>
+        <f aca="false">M23*Assumptions!$B$21</f>
+        <v>9000</v>
       </c>
       <c r="N24" s="6" t="n">
-        <f aca="false">Assumptions!$B$22</f>
-        <v>500</v>
+        <f aca="false">N23*Assumptions!$B$21</f>
+        <v>9000</v>
       </c>
       <c r="O24" s="6" t="n">
-        <f aca="false">Assumptions!$B$22</f>
-        <v>500</v>
+        <f aca="false">O23*Assumptions!$B$21</f>
+        <v>9000</v>
       </c>
       <c r="P24" s="6" t="n">
-        <f aca="false">Assumptions!$B$22</f>
-        <v>500</v>
+        <f aca="false">P23*Assumptions!$B$21</f>
+        <v>9000</v>
       </c>
       <c r="Q24" s="6" t="n">
-        <f aca="false">Assumptions!$B$22</f>
-        <v>500</v>
+        <f aca="false">Q23*Assumptions!$B$21</f>
+        <v>9000</v>
       </c>
       <c r="R24" s="6" t="n">
-        <f aca="false">Assumptions!$B$22</f>
-        <v>500</v>
+        <f aca="false">R23*Assumptions!$B$21</f>
+        <v>9000</v>
       </c>
       <c r="S24" s="6" t="n">
-        <f aca="false">Assumptions!$B$22</f>
-        <v>500</v>
+        <f aca="false">S23*Assumptions!$B$21</f>
+        <v>9000</v>
       </c>
       <c r="T24" s="6" t="n">
-        <f aca="false">Assumptions!$B$22</f>
-        <v>500</v>
+        <f aca="false">T23*Assumptions!$B$21</f>
+        <v>9000</v>
       </c>
       <c r="U24" s="6" t="n">
-        <f aca="false">Assumptions!$B$22</f>
-        <v>500</v>
+        <f aca="false">U23*Assumptions!$B$21</f>
+        <v>9000</v>
       </c>
       <c r="V24" s="6" t="n">
-        <f aca="false">Assumptions!$B$22</f>
-        <v>500</v>
+        <f aca="false">V23*Assumptions!$B$21</f>
+        <v>18000</v>
       </c>
       <c r="W24" s="6" t="n">
-        <f aca="false">Assumptions!$B$22</f>
-        <v>500</v>
+        <f aca="false">W23*Assumptions!$B$21</f>
+        <v>18000</v>
       </c>
       <c r="X24" s="6" t="n">
-        <f aca="false">Assumptions!$B$22</f>
-        <v>500</v>
+        <f aca="false">X23*Assumptions!$B$21</f>
+        <v>18000</v>
       </c>
       <c r="Y24" s="6" t="n">
-        <f aca="false">Assumptions!$B$22</f>
-        <v>500</v>
+        <f aca="false">Y23*Assumptions!$B$21</f>
+        <v>18000</v>
       </c>
       <c r="Z24" s="6" t="n">
         <f aca="false">SUM(B24:M24)</f>
-        <v>6000</v>
+        <v>36000</v>
       </c>
       <c r="AA24" s="6" t="n">
         <f aca="false">SUM(N24:Y24)</f>
-        <v>6000</v>
+        <v>144000</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="B25" s="6" t="n">
-        <f aca="false">Assumptions!$B$23</f>
-        <v>1200</v>
+        <f aca="false">Assumptions!$B$24</f>
+        <v>150</v>
       </c>
       <c r="C25" s="6" t="n">
-        <f aca="false">Assumptions!$B$23</f>
-        <v>1200</v>
+        <f aca="false">Assumptions!$B$24</f>
+        <v>150</v>
       </c>
       <c r="D25" s="6" t="n">
-        <f aca="false">Assumptions!$B$23</f>
-        <v>1200</v>
+        <f aca="false">Assumptions!$B$24</f>
+        <v>150</v>
       </c>
       <c r="E25" s="6" t="n">
-        <f aca="false">Assumptions!$B$23</f>
-        <v>1200</v>
+        <f aca="false">Assumptions!$B$24</f>
+        <v>150</v>
       </c>
       <c r="F25" s="6" t="n">
-        <f aca="false">Assumptions!$B$23</f>
-        <v>1200</v>
+        <f aca="false">Assumptions!$B$24</f>
+        <v>150</v>
       </c>
       <c r="G25" s="6" t="n">
-        <f aca="false">Assumptions!$B$23</f>
-        <v>1200</v>
+        <f aca="false">Assumptions!$B$24</f>
+        <v>150</v>
       </c>
       <c r="H25" s="6" t="n">
-        <f aca="false">Assumptions!$B$23</f>
-        <v>1200</v>
+        <f aca="false">Assumptions!$B$24</f>
+        <v>150</v>
       </c>
       <c r="I25" s="6" t="n">
-        <f aca="false">Assumptions!$B$23</f>
-        <v>1200</v>
+        <f aca="false">Assumptions!$B$24</f>
+        <v>150</v>
       </c>
       <c r="J25" s="6" t="n">
-        <f aca="false">Assumptions!$B$23</f>
-        <v>1200</v>
+        <f aca="false">Assumptions!$B$24</f>
+        <v>150</v>
       </c>
       <c r="K25" s="6" t="n">
-        <f aca="false">Assumptions!$B$23</f>
-        <v>1200</v>
+        <f aca="false">Assumptions!$B$24</f>
+        <v>150</v>
       </c>
       <c r="L25" s="6" t="n">
-        <f aca="false">Assumptions!$B$23</f>
-        <v>1200</v>
+        <f aca="false">Assumptions!$B$24</f>
+        <v>150</v>
       </c>
       <c r="M25" s="6" t="n">
-        <f aca="false">Assumptions!$B$23</f>
-        <v>1200</v>
+        <f aca="false">Assumptions!$B$24</f>
+        <v>150</v>
       </c>
       <c r="N25" s="6" t="n">
-        <f aca="false">Assumptions!$B$23</f>
-        <v>1200</v>
+        <f aca="false">Assumptions!$B$24</f>
+        <v>150</v>
       </c>
       <c r="O25" s="6" t="n">
-        <f aca="false">Assumptions!$B$23</f>
-        <v>1200</v>
+        <f aca="false">Assumptions!$B$24</f>
+        <v>150</v>
       </c>
       <c r="P25" s="6" t="n">
-        <f aca="false">Assumptions!$B$23</f>
-        <v>1200</v>
+        <f aca="false">Assumptions!$B$24</f>
+        <v>150</v>
       </c>
       <c r="Q25" s="6" t="n">
-        <f aca="false">Assumptions!$B$23</f>
-        <v>1200</v>
+        <f aca="false">Assumptions!$B$24</f>
+        <v>150</v>
       </c>
       <c r="R25" s="6" t="n">
-        <f aca="false">Assumptions!$B$23</f>
-        <v>1200</v>
+        <f aca="false">Assumptions!$B$24</f>
+        <v>150</v>
       </c>
       <c r="S25" s="6" t="n">
-        <f aca="false">Assumptions!$B$23</f>
-        <v>1200</v>
+        <f aca="false">Assumptions!$B$24</f>
+        <v>150</v>
       </c>
       <c r="T25" s="6" t="n">
-        <f aca="false">Assumptions!$B$23</f>
-        <v>1200</v>
+        <f aca="false">Assumptions!$B$24</f>
+        <v>150</v>
       </c>
       <c r="U25" s="6" t="n">
-        <f aca="false">Assumptions!$B$23</f>
-        <v>1200</v>
+        <f aca="false">Assumptions!$B$24</f>
+        <v>150</v>
       </c>
       <c r="V25" s="6" t="n">
-        <f aca="false">Assumptions!$B$23</f>
-        <v>1200</v>
+        <f aca="false">Assumptions!$B$24</f>
+        <v>150</v>
       </c>
       <c r="W25" s="6" t="n">
-        <f aca="false">Assumptions!$B$23</f>
-        <v>1200</v>
+        <f aca="false">Assumptions!$B$24</f>
+        <v>150</v>
       </c>
       <c r="X25" s="6" t="n">
-        <f aca="false">Assumptions!$B$23</f>
-        <v>1200</v>
+        <f aca="false">Assumptions!$B$24</f>
+        <v>150</v>
       </c>
       <c r="Y25" s="6" t="n">
-        <f aca="false">Assumptions!$B$23</f>
-        <v>1200</v>
+        <f aca="false">Assumptions!$B$24</f>
+        <v>150</v>
       </c>
       <c r="Z25" s="6" t="n">
         <f aca="false">SUM(B25:M25)</f>
-        <v>14400</v>
+        <v>1800</v>
       </c>
       <c r="AA25" s="6" t="n">
         <f aca="false">SUM(N25:Y25)</f>
-        <v>14400</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="B26" s="6" t="n">
-        <f aca="false">Assumptions!$B$24</f>
-        <v>7500</v>
+        <f aca="false">Assumptions!$B$25</f>
+        <v>500</v>
       </c>
       <c r="C26" s="6" t="n">
-        <f aca="false">Assumptions!$B$24</f>
-        <v>7500</v>
+        <f aca="false">Assumptions!$B$25</f>
+        <v>500</v>
       </c>
       <c r="D26" s="6" t="n">
-        <f aca="false">Assumptions!$B$24</f>
-        <v>7500</v>
+        <f aca="false">Assumptions!$B$25</f>
+        <v>500</v>
       </c>
       <c r="E26" s="6" t="n">
-        <f aca="false">Assumptions!$B$24</f>
-        <v>7500</v>
+        <f aca="false">Assumptions!$B$25</f>
+        <v>500</v>
       </c>
       <c r="F26" s="6" t="n">
-        <f aca="false">Assumptions!$B$24</f>
-        <v>7500</v>
+        <f aca="false">Assumptions!$B$25</f>
+        <v>500</v>
       </c>
       <c r="G26" s="6" t="n">
-        <f aca="false">Assumptions!$B$24</f>
-        <v>7500</v>
+        <f aca="false">Assumptions!$B$25</f>
+        <v>500</v>
       </c>
       <c r="H26" s="6" t="n">
-        <f aca="false">Assumptions!$B$24</f>
-        <v>7500</v>
+        <f aca="false">Assumptions!$B$25</f>
+        <v>500</v>
       </c>
       <c r="I26" s="6" t="n">
-        <f aca="false">Assumptions!$B$24</f>
-        <v>7500</v>
+        <f aca="false">Assumptions!$B$25</f>
+        <v>500</v>
       </c>
       <c r="J26" s="6" t="n">
-        <f aca="false">Assumptions!$B$24</f>
-        <v>7500</v>
+        <f aca="false">Assumptions!$B$25</f>
+        <v>500</v>
       </c>
       <c r="K26" s="6" t="n">
-        <f aca="false">Assumptions!$B$24</f>
-        <v>7500</v>
+        <f aca="false">Assumptions!$B$25</f>
+        <v>500</v>
       </c>
       <c r="L26" s="6" t="n">
-        <f aca="false">Assumptions!$B$24</f>
-        <v>7500</v>
+        <f aca="false">Assumptions!$B$25</f>
+        <v>500</v>
       </c>
       <c r="M26" s="6" t="n">
-        <f aca="false">Assumptions!$B$24</f>
-        <v>7500</v>
+        <f aca="false">Assumptions!$B$25</f>
+        <v>500</v>
       </c>
       <c r="N26" s="6" t="n">
-        <f aca="false">Assumptions!$B$24</f>
-        <v>7500</v>
+        <f aca="false">Assumptions!$B$25</f>
+        <v>500</v>
       </c>
       <c r="O26" s="6" t="n">
-        <f aca="false">Assumptions!$B$24</f>
-        <v>7500</v>
+        <f aca="false">Assumptions!$B$25</f>
+        <v>500</v>
       </c>
       <c r="P26" s="6" t="n">
-        <f aca="false">Assumptions!$B$24</f>
-        <v>7500</v>
+        <f aca="false">Assumptions!$B$25</f>
+        <v>500</v>
       </c>
       <c r="Q26" s="6" t="n">
-        <f aca="false">Assumptions!$B$24</f>
-        <v>7500</v>
+        <f aca="false">Assumptions!$B$25</f>
+        <v>500</v>
       </c>
       <c r="R26" s="6" t="n">
-        <f aca="false">Assumptions!$B$24</f>
-        <v>7500</v>
+        <f aca="false">Assumptions!$B$25</f>
+        <v>500</v>
       </c>
       <c r="S26" s="6" t="n">
-        <f aca="false">Assumptions!$B$24</f>
-        <v>7500</v>
+        <f aca="false">Assumptions!$B$25</f>
+        <v>500</v>
       </c>
       <c r="T26" s="6" t="n">
-        <f aca="false">Assumptions!$B$24</f>
-        <v>7500</v>
+        <f aca="false">Assumptions!$B$25</f>
+        <v>500</v>
       </c>
       <c r="U26" s="6" t="n">
-        <f aca="false">Assumptions!$B$24</f>
-        <v>7500</v>
+        <f aca="false">Assumptions!$B$25</f>
+        <v>500</v>
       </c>
       <c r="V26" s="6" t="n">
-        <f aca="false">Assumptions!$B$24</f>
-        <v>7500</v>
+        <f aca="false">Assumptions!$B$25</f>
+        <v>500</v>
       </c>
       <c r="W26" s="6" t="n">
-        <f aca="false">Assumptions!$B$24</f>
-        <v>7500</v>
+        <f aca="false">Assumptions!$B$25</f>
+        <v>500</v>
       </c>
       <c r="X26" s="6" t="n">
-        <f aca="false">Assumptions!$B$24</f>
-        <v>7500</v>
+        <f aca="false">Assumptions!$B$25</f>
+        <v>500</v>
       </c>
       <c r="Y26" s="6" t="n">
-        <f aca="false">Assumptions!$B$24</f>
-        <v>7500</v>
+        <f aca="false">Assumptions!$B$25</f>
+        <v>500</v>
       </c>
       <c r="Z26" s="6" t="n">
         <f aca="false">SUM(B26:M26)</f>
-        <v>90000</v>
+        <v>6000</v>
       </c>
       <c r="AA26" s="6" t="n">
         <f aca="false">SUM(N26:Y26)</f>
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="B27" s="6" t="n">
+        <f aca="false">Assumptions!$B$26</f>
+        <v>1200</v>
+      </c>
+      <c r="C27" s="6" t="n">
+        <f aca="false">Assumptions!$B$26</f>
+        <v>1200</v>
+      </c>
+      <c r="D27" s="6" t="n">
+        <f aca="false">Assumptions!$B$26</f>
+        <v>1200</v>
+      </c>
+      <c r="E27" s="6" t="n">
+        <f aca="false">Assumptions!$B$26</f>
+        <v>1200</v>
+      </c>
+      <c r="F27" s="6" t="n">
+        <f aca="false">Assumptions!$B$26</f>
+        <v>1200</v>
+      </c>
+      <c r="G27" s="6" t="n">
+        <f aca="false">Assumptions!$B$26</f>
+        <v>1200</v>
+      </c>
+      <c r="H27" s="6" t="n">
+        <f aca="false">Assumptions!$B$26</f>
+        <v>1200</v>
+      </c>
+      <c r="I27" s="6" t="n">
+        <f aca="false">Assumptions!$B$26</f>
+        <v>1200</v>
+      </c>
+      <c r="J27" s="6" t="n">
+        <f aca="false">Assumptions!$B$26</f>
+        <v>1200</v>
+      </c>
+      <c r="K27" s="6" t="n">
+        <f aca="false">Assumptions!$B$26</f>
+        <v>1200</v>
+      </c>
+      <c r="L27" s="6" t="n">
+        <f aca="false">Assumptions!$B$26</f>
+        <v>1200</v>
+      </c>
+      <c r="M27" s="6" t="n">
+        <f aca="false">Assumptions!$B$26</f>
+        <v>1200</v>
+      </c>
+      <c r="N27" s="6" t="n">
+        <f aca="false">Assumptions!$B$26</f>
+        <v>1200</v>
+      </c>
+      <c r="O27" s="6" t="n">
+        <f aca="false">Assumptions!$B$26</f>
+        <v>1200</v>
+      </c>
+      <c r="P27" s="6" t="n">
+        <f aca="false">Assumptions!$B$26</f>
+        <v>1200</v>
+      </c>
+      <c r="Q27" s="6" t="n">
+        <f aca="false">Assumptions!$B$26</f>
+        <v>1200</v>
+      </c>
+      <c r="R27" s="6" t="n">
+        <f aca="false">Assumptions!$B$26</f>
+        <v>1200</v>
+      </c>
+      <c r="S27" s="6" t="n">
+        <f aca="false">Assumptions!$B$26</f>
+        <v>1200</v>
+      </c>
+      <c r="T27" s="6" t="n">
+        <f aca="false">Assumptions!$B$26</f>
+        <v>1200</v>
+      </c>
+      <c r="U27" s="6" t="n">
+        <f aca="false">Assumptions!$B$26</f>
+        <v>1200</v>
+      </c>
+      <c r="V27" s="6" t="n">
+        <f aca="false">Assumptions!$B$26</f>
+        <v>1200</v>
+      </c>
+      <c r="W27" s="6" t="n">
+        <f aca="false">Assumptions!$B$26</f>
+        <v>1200</v>
+      </c>
+      <c r="X27" s="6" t="n">
+        <f aca="false">Assumptions!$B$26</f>
+        <v>1200</v>
+      </c>
+      <c r="Y27" s="6" t="n">
+        <f aca="false">Assumptions!$B$26</f>
+        <v>1200</v>
+      </c>
+      <c r="Z27" s="6" t="n">
+        <f aca="false">SUM(B27:M27)</f>
+        <v>14400</v>
+      </c>
+      <c r="AA27" s="6" t="n">
+        <f aca="false">SUM(N27:Y27)</f>
+        <v>14400</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="B28" s="6" t="n">
+        <f aca="false">Assumptions!$B$27</f>
+        <v>7500</v>
+      </c>
+      <c r="C28" s="6" t="n">
+        <f aca="false">Assumptions!$B$27</f>
+        <v>7500</v>
+      </c>
+      <c r="D28" s="6" t="n">
+        <f aca="false">Assumptions!$B$27</f>
+        <v>7500</v>
+      </c>
+      <c r="E28" s="6" t="n">
+        <f aca="false">Assumptions!$B$27</f>
+        <v>7500</v>
+      </c>
+      <c r="F28" s="6" t="n">
+        <f aca="false">Assumptions!$B$27</f>
+        <v>7500</v>
+      </c>
+      <c r="G28" s="6" t="n">
+        <f aca="false">Assumptions!$B$27</f>
+        <v>7500</v>
+      </c>
+      <c r="H28" s="6" t="n">
+        <f aca="false">Assumptions!$B$27</f>
+        <v>7500</v>
+      </c>
+      <c r="I28" s="6" t="n">
+        <f aca="false">Assumptions!$B$27</f>
+        <v>7500</v>
+      </c>
+      <c r="J28" s="6" t="n">
+        <f aca="false">Assumptions!$B$27</f>
+        <v>7500</v>
+      </c>
+      <c r="K28" s="6" t="n">
+        <f aca="false">Assumptions!$B$27</f>
+        <v>7500</v>
+      </c>
+      <c r="L28" s="6" t="n">
+        <f aca="false">Assumptions!$B$27</f>
+        <v>7500</v>
+      </c>
+      <c r="M28" s="6" t="n">
+        <f aca="false">Assumptions!$B$27</f>
+        <v>7500</v>
+      </c>
+      <c r="N28" s="6" t="n">
+        <f aca="false">Assumptions!$B$27</f>
+        <v>7500</v>
+      </c>
+      <c r="O28" s="6" t="n">
+        <f aca="false">Assumptions!$B$27</f>
+        <v>7500</v>
+      </c>
+      <c r="P28" s="6" t="n">
+        <f aca="false">Assumptions!$B$27</f>
+        <v>7500</v>
+      </c>
+      <c r="Q28" s="6" t="n">
+        <f aca="false">Assumptions!$B$27</f>
+        <v>7500</v>
+      </c>
+      <c r="R28" s="6" t="n">
+        <f aca="false">Assumptions!$B$27</f>
+        <v>7500</v>
+      </c>
+      <c r="S28" s="6" t="n">
+        <f aca="false">Assumptions!$B$27</f>
+        <v>7500</v>
+      </c>
+      <c r="T28" s="6" t="n">
+        <f aca="false">Assumptions!$B$27</f>
+        <v>7500</v>
+      </c>
+      <c r="U28" s="6" t="n">
+        <f aca="false">Assumptions!$B$27</f>
+        <v>7500</v>
+      </c>
+      <c r="V28" s="6" t="n">
+        <f aca="false">Assumptions!$B$27</f>
+        <v>7500</v>
+      </c>
+      <c r="W28" s="6" t="n">
+        <f aca="false">Assumptions!$B$27</f>
+        <v>7500</v>
+      </c>
+      <c r="X28" s="6" t="n">
+        <f aca="false">Assumptions!$B$27</f>
+        <v>7500</v>
+      </c>
+      <c r="Y28" s="6" t="n">
+        <f aca="false">Assumptions!$B$27</f>
+        <v>7500</v>
+      </c>
+      <c r="Z28" s="6" t="n">
+        <f aca="false">SUM(B28:M28)</f>
         <v>90000</v>
       </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="B27" s="7" t="n">
-        <f aca="false">SUM(B21:B26)</f>
-        <v>10275</v>
-      </c>
-      <c r="C27" s="7" t="n">
-        <f aca="false">SUM(C21:C26)</f>
-        <v>10325</v>
-      </c>
-      <c r="D27" s="7" t="n">
-        <f aca="false">SUM(D21:D26)</f>
-        <v>10375</v>
-      </c>
-      <c r="E27" s="7" t="n">
-        <f aca="false">SUM(E21:E26)</f>
-        <v>10425</v>
-      </c>
-      <c r="F27" s="7" t="n">
-        <f aca="false">SUM(F21:F26)</f>
-        <v>10475</v>
-      </c>
-      <c r="G27" s="7" t="n">
-        <f aca="false">SUM(G21:G26)</f>
-        <v>10525</v>
-      </c>
-      <c r="H27" s="7" t="n">
-        <f aca="false">SUM(H21:H26)</f>
-        <v>15200</v>
-      </c>
-      <c r="I27" s="7" t="n">
-        <f aca="false">SUM(I21:I26)</f>
-        <v>18275</v>
-      </c>
-      <c r="J27" s="7" t="n">
-        <f aca="false">SUM(J21:J26)</f>
-        <v>22425</v>
-      </c>
-      <c r="K27" s="7" t="n">
-        <f aca="false">SUM(K21:K26)</f>
-        <v>26775</v>
-      </c>
-      <c r="L27" s="7" t="n">
-        <f aca="false">SUM(L21:L26)</f>
-        <v>31325</v>
-      </c>
-      <c r="M27" s="7" t="n">
-        <f aca="false">SUM(M21:M26)</f>
-        <v>38850</v>
-      </c>
-      <c r="N27" s="7" t="n">
-        <f aca="false">SUM(N21:N26)</f>
-        <v>28200</v>
-      </c>
-      <c r="O27" s="7" t="n">
-        <f aca="false">SUM(O21:O26)</f>
-        <v>28896.5</v>
-      </c>
-      <c r="P27" s="7" t="n">
-        <f aca="false">SUM(P21:P26)</f>
-        <v>29586.035</v>
-      </c>
-      <c r="Q27" s="7" t="n">
-        <f aca="false">SUM(Q21:Q26)</f>
-        <v>30268.67465</v>
-      </c>
-      <c r="R27" s="7" t="n">
-        <f aca="false">SUM(R21:R26)</f>
-        <v>30944.4879035</v>
-      </c>
-      <c r="S27" s="7" t="n">
-        <f aca="false">SUM(S21:S26)</f>
-        <v>31613.543024465</v>
-      </c>
-      <c r="T27" s="7" t="n">
-        <f aca="false">SUM(T21:T26)</f>
-        <v>32275.9075942204</v>
-      </c>
-      <c r="U27" s="7" t="n">
-        <f aca="false">SUM(U21:U26)</f>
-        <v>32931.6485182782</v>
-      </c>
-      <c r="V27" s="7" t="n">
-        <f aca="false">SUM(V21:V26)</f>
-        <v>33580.8320330954</v>
-      </c>
-      <c r="W27" s="7" t="n">
-        <f aca="false">SUM(W21:W26)</f>
-        <v>34223.5237127644</v>
-      </c>
-      <c r="X27" s="7" t="n">
-        <f aca="false">SUM(X21:X26)</f>
-        <v>34859.7884756368</v>
-      </c>
-      <c r="Y27" s="7" t="n">
-        <f aca="false">SUM(Y21:Y26)</f>
-        <v>35489.6905908804</v>
-      </c>
-      <c r="Z27" s="7" t="n">
-        <f aca="false">SUM(B27:M27)</f>
-        <v>215250</v>
-      </c>
-      <c r="AA27" s="7" t="n">
-        <f aca="false">SUM(N27:Y27)</f>
-        <v>382870.63150284</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="B28" s="7" t="n">
-        <f aca="false">B18-B27</f>
-        <v>-10026</v>
-      </c>
-      <c r="C28" s="7" t="n">
-        <f aca="false">C18-C27</f>
-        <v>-9578</v>
-      </c>
-      <c r="D28" s="7" t="n">
-        <f aca="false">D18-D27</f>
-        <v>-9130</v>
-      </c>
-      <c r="E28" s="7" t="n">
-        <f aca="false">E18-E27</f>
-        <v>-8682</v>
-      </c>
-      <c r="F28" s="7" t="n">
-        <f aca="false">F18-F27</f>
-        <v>-8234</v>
-      </c>
-      <c r="G28" s="7" t="n">
-        <f aca="false">G18-G27</f>
-        <v>-7786</v>
-      </c>
-      <c r="H28" s="7" t="n">
-        <f aca="false">H18-H27</f>
-        <v>-10718</v>
-      </c>
-      <c r="I28" s="7" t="n">
-        <f aca="false">I18-I27</f>
-        <v>-10058</v>
-      </c>
-      <c r="J28" s="7" t="n">
-        <f aca="false">J18-J27</f>
-        <v>-8730</v>
-      </c>
-      <c r="K28" s="7" t="n">
-        <f aca="false">K18-K27</f>
-        <v>-5610</v>
-      </c>
-      <c r="L28" s="7" t="n">
-        <f aca="false">L18-L27</f>
-        <v>-698</v>
-      </c>
-      <c r="M28" s="7" t="n">
-        <f aca="false">M18-M27</f>
-        <v>3978</v>
-      </c>
-      <c r="N28" s="7" t="n">
-        <f aca="false">N18-N27</f>
-        <v>25086</v>
-      </c>
-      <c r="O28" s="7" t="n">
-        <f aca="false">O18-O27</f>
-        <v>31326.64</v>
-      </c>
-      <c r="P28" s="7" t="n">
-        <f aca="false">P18-P27</f>
-        <v>37504.8736</v>
-      </c>
-      <c r="Q28" s="7" t="n">
-        <f aca="false">Q18-Q27</f>
-        <v>43621.324864</v>
-      </c>
-      <c r="R28" s="7" t="n">
-        <f aca="false">R18-R27</f>
-        <v>49676.61161536</v>
-      </c>
-      <c r="S28" s="7" t="n">
-        <f aca="false">S18-S27</f>
-        <v>55671.3454992064</v>
-      </c>
-      <c r="T28" s="7" t="n">
-        <f aca="false">T18-T27</f>
-        <v>61606.1320442143</v>
-      </c>
-      <c r="U28" s="7" t="n">
-        <f aca="false">U18-U27</f>
-        <v>67481.5707237722</v>
-      </c>
-      <c r="V28" s="7" t="n">
-        <f aca="false">V18-V27</f>
-        <v>73298.2550165345</v>
-      </c>
-      <c r="W28" s="7" t="n">
-        <f aca="false">W18-W27</f>
-        <v>79056.7724663691</v>
-      </c>
-      <c r="X28" s="7" t="n">
-        <f aca="false">X18-X27</f>
-        <v>84757.7047417054</v>
-      </c>
-      <c r="Y28" s="7" t="n">
-        <f aca="false">Y18-Y27</f>
-        <v>90401.6276942884</v>
-      </c>
-      <c r="Z28" s="7" t="n">
-        <f aca="false">SUM(B28:M28)</f>
-        <v>-85272</v>
-      </c>
-      <c r="AA28" s="7" t="n">
+      <c r="AA28" s="6" t="n">
         <f aca="false">SUM(N28:Y28)</f>
-        <v>699488.85826545</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="s">
-        <v>96</v>
-      </c>
-      <c r="B29" s="6" t="n">
-        <f aca="false">MAX(0,Assumptions!$B$25*MAX(0,SUM($B28:B28))-0)</f>
-        <v>0</v>
-      </c>
-      <c r="C29" s="6" t="n">
-        <f aca="false">MAX(0,Assumptions!$B$25*MAX(0,SUM($B28:C28))-SUM($B29:B29))</f>
-        <v>0</v>
-      </c>
-      <c r="D29" s="6" t="n">
-        <f aca="false">MAX(0,Assumptions!$B$25*MAX(0,SUM($B28:D28))-SUM($B29:C29))</f>
-        <v>0</v>
-      </c>
-      <c r="E29" s="6" t="n">
-        <f aca="false">MAX(0,Assumptions!$B$25*MAX(0,SUM($B28:E28))-SUM($B29:D29))</f>
-        <v>0</v>
-      </c>
-      <c r="F29" s="6" t="n">
-        <f aca="false">MAX(0,Assumptions!$B$25*MAX(0,SUM($B28:F28))-SUM($B29:E29))</f>
-        <v>0</v>
-      </c>
-      <c r="G29" s="6" t="n">
-        <f aca="false">MAX(0,Assumptions!$B$25*MAX(0,SUM($B28:G28))-SUM($B29:F29))</f>
-        <v>0</v>
-      </c>
-      <c r="H29" s="6" t="n">
-        <f aca="false">MAX(0,Assumptions!$B$25*MAX(0,SUM($B28:H28))-SUM($B29:G29))</f>
-        <v>0</v>
-      </c>
-      <c r="I29" s="6" t="n">
-        <f aca="false">MAX(0,Assumptions!$B$25*MAX(0,SUM($B28:I28))-SUM($B29:H29))</f>
-        <v>0</v>
-      </c>
-      <c r="J29" s="6" t="n">
-        <f aca="false">MAX(0,Assumptions!$B$25*MAX(0,SUM($B28:J28))-SUM($B29:I29))</f>
-        <v>0</v>
-      </c>
-      <c r="K29" s="6" t="n">
-        <f aca="false">MAX(0,Assumptions!$B$25*MAX(0,SUM($B28:K28))-SUM($B29:J29))</f>
-        <v>0</v>
-      </c>
-      <c r="L29" s="6" t="n">
-        <f aca="false">MAX(0,Assumptions!$B$25*MAX(0,SUM($B28:L28))-SUM($B29:K29))</f>
-        <v>0</v>
-      </c>
-      <c r="M29" s="6" t="n">
-        <f aca="false">MAX(0,Assumptions!$B$25*MAX(0,SUM($B28:M28))-SUM($B29:L29))</f>
-        <v>0</v>
-      </c>
-      <c r="N29" s="6" t="n">
-        <f aca="false">MAX(0,Assumptions!$B$25*MAX(0,SUM($B28:N28))-SUM($B29:M29))</f>
-        <v>0</v>
-      </c>
-      <c r="O29" s="6" t="n">
-        <f aca="false">MAX(0,Assumptions!$B$25*MAX(0,SUM($B28:O28))-SUM($B29:N29))</f>
-        <v>0</v>
-      </c>
-      <c r="P29" s="6" t="n">
-        <f aca="false">MAX(0,Assumptions!$B$25*MAX(0,SUM($B28:P28))-SUM($B29:O29))</f>
-        <v>2161.3784</v>
-      </c>
-      <c r="Q29" s="6" t="n">
-        <f aca="false">MAX(0,Assumptions!$B$25*MAX(0,SUM($B28:Q28))-SUM($B29:P29))</f>
-        <v>10905.331216</v>
-      </c>
-      <c r="R29" s="6" t="n">
-        <f aca="false">MAX(0,Assumptions!$B$25*MAX(0,SUM($B28:R28))-SUM($B29:Q29))</f>
-        <v>12419.15290384</v>
-      </c>
-      <c r="S29" s="6" t="n">
-        <f aca="false">MAX(0,Assumptions!$B$25*MAX(0,SUM($B28:S28))-SUM($B29:R29))</f>
-        <v>13917.8363748016</v>
-      </c>
-      <c r="T29" s="6" t="n">
-        <f aca="false">MAX(0,Assumptions!$B$25*MAX(0,SUM($B28:T28))-SUM($B29:S29))</f>
-        <v>15401.5330110536</v>
-      </c>
-      <c r="U29" s="6" t="n">
-        <f aca="false">MAX(0,Assumptions!$B$25*MAX(0,SUM($B28:U28))-SUM($B29:T29))</f>
-        <v>16870.392680943</v>
-      </c>
-      <c r="V29" s="6" t="n">
-        <f aca="false">MAX(0,Assumptions!$B$25*MAX(0,SUM($B28:V28))-SUM($B29:U29))</f>
-        <v>18324.5637541336</v>
-      </c>
-      <c r="W29" s="6" t="n">
-        <f aca="false">MAX(0,Assumptions!$B$25*MAX(0,SUM($B28:W28))-SUM($B29:V29))</f>
-        <v>19764.1931165923</v>
-      </c>
-      <c r="X29" s="6" t="n">
-        <f aca="false">MAX(0,Assumptions!$B$25*MAX(0,SUM($B28:X28))-SUM($B29:W29))</f>
-        <v>21189.4261854264</v>
-      </c>
-      <c r="Y29" s="6" t="n">
-        <f aca="false">MAX(0,Assumptions!$B$25*MAX(0,SUM($B28:Y28))-SUM($B29:X29))</f>
-        <v>22600.4069235721</v>
-      </c>
-      <c r="Z29" s="6" t="n">
+      <c r="A29" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B29" s="7" t="n">
+        <f aca="false">SUM(B21:B28)</f>
+        <v>9755</v>
+      </c>
+      <c r="C29" s="7" t="n">
+        <f aca="false">SUM(C21:C28)</f>
+        <v>9765</v>
+      </c>
+      <c r="D29" s="7" t="n">
+        <f aca="false">SUM(D21:D28)</f>
+        <v>9775</v>
+      </c>
+      <c r="E29" s="7" t="n">
+        <f aca="false">SUM(E21:E28)</f>
+        <v>9785</v>
+      </c>
+      <c r="F29" s="7" t="n">
+        <f aca="false">SUM(F21:F28)</f>
+        <v>9795</v>
+      </c>
+      <c r="G29" s="7" t="n">
+        <f aca="false">SUM(G21:G28)</f>
+        <v>9805</v>
+      </c>
+      <c r="H29" s="7" t="n">
+        <f aca="false">SUM(H21:H28)</f>
+        <v>11840</v>
+      </c>
+      <c r="I29" s="7" t="n">
+        <f aca="false">SUM(I21:I28)</f>
+        <v>13115</v>
+      </c>
+      <c r="J29" s="7" t="n">
+        <f aca="false">SUM(J21:J28)</f>
+        <v>23826</v>
+      </c>
+      <c r="K29" s="7" t="n">
+        <f aca="false">SUM(K21:K28)</f>
+        <v>25576</v>
+      </c>
+      <c r="L29" s="7" t="n">
+        <f aca="false">SUM(L21:L28)</f>
+        <v>27366</v>
+      </c>
+      <c r="M29" s="7" t="n">
+        <f aca="false">SUM(M21:M28)</f>
+        <v>30411</v>
+      </c>
+      <c r="N29" s="7" t="n">
+        <f aca="false">SUM(N21:N28)</f>
+        <v>25421</v>
+      </c>
+      <c r="O29" s="7" t="n">
+        <f aca="false">SUM(O21:O28)</f>
+        <v>25560.3</v>
+      </c>
+      <c r="P29" s="7" t="n">
+        <f aca="false">SUM(P21:P28)</f>
+        <v>25698.207</v>
+      </c>
+      <c r="Q29" s="7" t="n">
+        <f aca="false">SUM(Q21:Q28)</f>
+        <v>25834.73493</v>
+      </c>
+      <c r="R29" s="7" t="n">
+        <f aca="false">SUM(R21:R28)</f>
+        <v>25969.8975807</v>
+      </c>
+      <c r="S29" s="7" t="n">
+        <f aca="false">SUM(S21:S28)</f>
+        <v>26103.708604893</v>
+      </c>
+      <c r="T29" s="7" t="n">
+        <f aca="false">SUM(T21:T28)</f>
+        <v>26236.1815188441</v>
+      </c>
+      <c r="U29" s="7" t="n">
+        <f aca="false">SUM(U21:U28)</f>
+        <v>26367.3297036556</v>
+      </c>
+      <c r="V29" s="7" t="n">
+        <f aca="false">SUM(V21:V28)</f>
+        <v>35498.1664066191</v>
+      </c>
+      <c r="W29" s="7" t="n">
+        <f aca="false">SUM(W21:W28)</f>
+        <v>35626.7047425529</v>
+      </c>
+      <c r="X29" s="7" t="n">
+        <f aca="false">SUM(X21:X28)</f>
+        <v>35753.9576951274</v>
+      </c>
+      <c r="Y29" s="7" t="n">
+        <f aca="false">SUM(Y21:Y28)</f>
+        <v>35879.9381181761</v>
+      </c>
+      <c r="Z29" s="7" t="n">
         <f aca="false">SUM(B29:M29)</f>
-        <v>0</v>
-      </c>
-      <c r="AA29" s="6" t="n">
+        <v>190814</v>
+      </c>
+      <c r="AA29" s="7" t="n">
         <f aca="false">SUM(N29:Y29)</f>
-        <v>153554.214566363</v>
+        <v>349950.126300568</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B30" s="7" t="n">
-        <f aca="false">B28-B29</f>
-        <v>-10026</v>
+        <f aca="false">B18-B29</f>
+        <v>-9506</v>
       </c>
       <c r="C30" s="7" t="n">
-        <f aca="false">C28-C29</f>
-        <v>-9578</v>
+        <f aca="false">C18-C29</f>
+        <v>-9018</v>
       </c>
       <c r="D30" s="7" t="n">
-        <f aca="false">D28-D29</f>
-        <v>-9130</v>
+        <f aca="false">D18-D29</f>
+        <v>-8530</v>
       </c>
       <c r="E30" s="7" t="n">
-        <f aca="false">E28-E29</f>
-        <v>-8682</v>
+        <f aca="false">E18-E29</f>
+        <v>-8042</v>
       </c>
       <c r="F30" s="7" t="n">
-        <f aca="false">F28-F29</f>
-        <v>-8234</v>
+        <f aca="false">F18-F29</f>
+        <v>-7554</v>
       </c>
       <c r="G30" s="7" t="n">
-        <f aca="false">G28-G29</f>
-        <v>-7786</v>
+        <f aca="false">G18-G29</f>
+        <v>-7066</v>
       </c>
       <c r="H30" s="7" t="n">
-        <f aca="false">H28-H29</f>
-        <v>-10718</v>
+        <f aca="false">H18-H29</f>
+        <v>-7358</v>
       </c>
       <c r="I30" s="7" t="n">
-        <f aca="false">I28-I29</f>
-        <v>-10058</v>
+        <f aca="false">I18-I29</f>
+        <v>-4898</v>
       </c>
       <c r="J30" s="7" t="n">
-        <f aca="false">J28-J29</f>
-        <v>-8730</v>
+        <f aca="false">J18-J29</f>
+        <v>-10131</v>
       </c>
       <c r="K30" s="7" t="n">
-        <f aca="false">K28-K29</f>
-        <v>-5610</v>
+        <f aca="false">K18-K29</f>
+        <v>-4411</v>
       </c>
       <c r="L30" s="7" t="n">
-        <f aca="false">L28-L29</f>
-        <v>-698</v>
+        <f aca="false">L18-L29</f>
+        <v>3261</v>
       </c>
       <c r="M30" s="7" t="n">
-        <f aca="false">M28-M29</f>
-        <v>3978</v>
+        <f aca="false">M18-M29</f>
+        <v>12417</v>
       </c>
       <c r="N30" s="7" t="n">
-        <f aca="false">N28-N29</f>
-        <v>25086</v>
+        <f aca="false">N18-N29</f>
+        <v>27865</v>
       </c>
       <c r="O30" s="7" t="n">
-        <f aca="false">O28-O29</f>
-        <v>31326.64</v>
+        <f aca="false">O18-O29</f>
+        <v>34662.84</v>
       </c>
       <c r="P30" s="7" t="n">
-        <f aca="false">P28-P29</f>
-        <v>35343.4952</v>
+        <f aca="false">P18-P29</f>
+        <v>41392.7016</v>
       </c>
       <c r="Q30" s="7" t="n">
-        <f aca="false">Q28-Q29</f>
-        <v>32715.993648</v>
+        <f aca="false">Q18-Q29</f>
+        <v>48055.264584</v>
       </c>
       <c r="R30" s="7" t="n">
-        <f aca="false">R28-R29</f>
-        <v>37257.45871152</v>
+        <f aca="false">R18-R29</f>
+        <v>54651.20193816</v>
       </c>
       <c r="S30" s="7" t="n">
-        <f aca="false">S28-S29</f>
-        <v>41753.5091244048</v>
+        <f aca="false">S18-S29</f>
+        <v>61181.1799187784</v>
       </c>
       <c r="T30" s="7" t="n">
-        <f aca="false">T28-T29</f>
-        <v>46204.5990331607</v>
+        <f aca="false">T18-T29</f>
+        <v>67645.8581195906</v>
       </c>
       <c r="U30" s="7" t="n">
-        <f aca="false">U28-U29</f>
-        <v>50611.1780428292</v>
+        <f aca="false">U18-U29</f>
+        <v>74045.8895383947</v>
       </c>
       <c r="V30" s="7" t="n">
-        <f aca="false">V28-V29</f>
-        <v>54973.6912624009</v>
+        <f aca="false">V18-V29</f>
+        <v>71380.9206430108</v>
       </c>
       <c r="W30" s="7" t="n">
-        <f aca="false">W28-W29</f>
-        <v>59292.5793497768</v>
+        <f aca="false">W18-W29</f>
+        <v>77653.5914365807</v>
       </c>
       <c r="X30" s="7" t="n">
-        <f aca="false">X28-X29</f>
-        <v>63568.2785562791</v>
+        <f aca="false">X18-X29</f>
+        <v>83863.5355222149</v>
       </c>
       <c r="Y30" s="7" t="n">
-        <f aca="false">Y28-Y29</f>
-        <v>67801.2207707163</v>
+        <f aca="false">Y18-Y29</f>
+        <v>90011.3801669927</v>
       </c>
       <c r="Z30" s="7" t="n">
         <f aca="false">SUM(B30:M30)</f>
-        <v>-85272</v>
+        <v>-60836</v>
       </c>
       <c r="AA30" s="7" t="n">
         <f aca="false">SUM(N30:Y30)</f>
-        <v>545934.643699088</v>
+        <v>732409.363467723</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="B31" s="6" t="n">
-        <f aca="false">SUM($B30:B30)</f>
-        <v>-10026</v>
+        <f aca="false">MAX(0,Assumptions!$B$28*MAX(0,SUM($B30:B30))-0)</f>
+        <v>0</v>
       </c>
       <c r="C31" s="6" t="n">
-        <f aca="false">SUM($B30:C30)</f>
-        <v>-19604</v>
+        <f aca="false">MAX(0,Assumptions!$B$28*MAX(0,SUM($B30:C30))-SUM($B31:B31))</f>
+        <v>0</v>
       </c>
       <c r="D31" s="6" t="n">
-        <f aca="false">SUM($B30:D30)</f>
-        <v>-28734</v>
+        <f aca="false">MAX(0,Assumptions!$B$28*MAX(0,SUM($B30:D30))-SUM($B31:C31))</f>
+        <v>0</v>
       </c>
       <c r="E31" s="6" t="n">
-        <f aca="false">SUM($B30:E30)</f>
-        <v>-37416</v>
+        <f aca="false">MAX(0,Assumptions!$B$28*MAX(0,SUM($B30:E30))-SUM($B31:D31))</f>
+        <v>0</v>
       </c>
       <c r="F31" s="6" t="n">
-        <f aca="false">SUM($B30:F30)</f>
-        <v>-45650</v>
+        <f aca="false">MAX(0,Assumptions!$B$28*MAX(0,SUM($B30:F30))-SUM($B31:E31))</f>
+        <v>0</v>
       </c>
       <c r="G31" s="6" t="n">
-        <f aca="false">SUM($B30:G30)</f>
-        <v>-53436</v>
+        <f aca="false">MAX(0,Assumptions!$B$28*MAX(0,SUM($B30:G30))-SUM($B31:F31))</f>
+        <v>0</v>
       </c>
       <c r="H31" s="6" t="n">
-        <f aca="false">SUM($B30:H30)</f>
-        <v>-64154</v>
+        <f aca="false">MAX(0,Assumptions!$B$28*MAX(0,SUM($B30:H30))-SUM($B31:G31))</f>
+        <v>0</v>
       </c>
       <c r="I31" s="6" t="n">
-        <f aca="false">SUM($B30:I30)</f>
-        <v>-74212</v>
+        <f aca="false">MAX(0,Assumptions!$B$28*MAX(0,SUM($B30:I30))-SUM($B31:H31))</f>
+        <v>0</v>
       </c>
       <c r="J31" s="6" t="n">
-        <f aca="false">SUM($B30:J30)</f>
-        <v>-82942</v>
+        <f aca="false">MAX(0,Assumptions!$B$28*MAX(0,SUM($B30:J30))-SUM($B31:I31))</f>
+        <v>0</v>
       </c>
       <c r="K31" s="6" t="n">
-        <f aca="false">SUM($B30:K30)</f>
-        <v>-88552</v>
+        <f aca="false">MAX(0,Assumptions!$B$28*MAX(0,SUM($B30:K30))-SUM($B31:J31))</f>
+        <v>0</v>
       </c>
       <c r="L31" s="6" t="n">
-        <f aca="false">SUM($B30:L30)</f>
-        <v>-89250</v>
+        <f aca="false">MAX(0,Assumptions!$B$28*MAX(0,SUM($B30:L30))-SUM($B31:K31))</f>
+        <v>0</v>
       </c>
       <c r="M31" s="6" t="n">
-        <f aca="false">SUM($B30:M30)</f>
-        <v>-85272</v>
+        <f aca="false">MAX(0,Assumptions!$B$28*MAX(0,SUM($B30:M30))-SUM($B31:L31))</f>
+        <v>0</v>
       </c>
       <c r="N31" s="6" t="n">
-        <f aca="false">SUM($B30:N30)</f>
-        <v>-60186</v>
+        <f aca="false">MAX(0,Assumptions!$B$28*MAX(0,SUM($B30:N30))-SUM($B31:M31))</f>
+        <v>0</v>
       </c>
       <c r="O31" s="6" t="n">
-        <f aca="false">SUM($B30:O30)</f>
-        <v>-28859.36</v>
+        <f aca="false">MAX(0,Assumptions!$B$28*MAX(0,SUM($B30:O30))-SUM($B31:N31))</f>
+        <v>422.960000000003</v>
       </c>
       <c r="P31" s="6" t="n">
-        <f aca="false">SUM($B30:P30)</f>
-        <v>6484.1352</v>
+        <f aca="false">MAX(0,Assumptions!$B$28*MAX(0,SUM($B30:P30))-SUM($B31:O31))</f>
+        <v>10348.1754</v>
       </c>
       <c r="Q31" s="6" t="n">
-        <f aca="false">SUM($B30:Q30)</f>
-        <v>39200.128848</v>
+        <f aca="false">MAX(0,Assumptions!$B$28*MAX(0,SUM($B30:Q30))-SUM($B31:P31))</f>
+        <v>12013.816146</v>
       </c>
       <c r="R31" s="6" t="n">
-        <f aca="false">SUM($B30:R30)</f>
-        <v>76457.58755952</v>
+        <f aca="false">MAX(0,Assumptions!$B$28*MAX(0,SUM($B30:R30))-SUM($B31:Q31))</f>
+        <v>13662.80048454</v>
       </c>
       <c r="S31" s="6" t="n">
-        <f aca="false">SUM($B30:S30)</f>
-        <v>118211.096683925</v>
+        <f aca="false">MAX(0,Assumptions!$B$28*MAX(0,SUM($B30:S30))-SUM($B31:R31))</f>
+        <v>15295.2949796946</v>
       </c>
       <c r="T31" s="6" t="n">
-        <f aca="false">SUM($B30:T30)</f>
-        <v>164415.695717086</v>
+        <f aca="false">MAX(0,Assumptions!$B$28*MAX(0,SUM($B30:T30))-SUM($B31:S31))</f>
+        <v>16911.4645298977</v>
       </c>
       <c r="U31" s="6" t="n">
-        <f aca="false">SUM($B30:U30)</f>
-        <v>215026.873759915</v>
+        <f aca="false">MAX(0,Assumptions!$B$28*MAX(0,SUM($B30:U30))-SUM($B31:T31))</f>
+        <v>18511.4723845987</v>
       </c>
       <c r="V31" s="6" t="n">
-        <f aca="false">SUM($B30:V30)</f>
-        <v>270000.565022316</v>
+        <f aca="false">MAX(0,Assumptions!$B$28*MAX(0,SUM($B30:V30))-SUM($B31:U31))</f>
+        <v>17845.2301607527</v>
       </c>
       <c r="W31" s="6" t="n">
-        <f aca="false">SUM($B30:W30)</f>
-        <v>329293.144372092</v>
+        <f aca="false">MAX(0,Assumptions!$B$28*MAX(0,SUM($B30:W30))-SUM($B31:V31))</f>
+        <v>19413.3978591452</v>
       </c>
       <c r="X31" s="6" t="n">
-        <f aca="false">SUM($B30:X30)</f>
-        <v>392861.422928371</v>
+        <f aca="false">MAX(0,Assumptions!$B$28*MAX(0,SUM($B30:X30))-SUM($B31:W31))</f>
+        <v>20965.8838805537</v>
       </c>
       <c r="Y31" s="6" t="n">
-        <f aca="false">SUM($B30:Y30)</f>
-        <v>460662.643699088</v>
+        <f aca="false">MAX(0,Assumptions!$B$28*MAX(0,SUM($B30:Y30))-SUM($B31:X31))</f>
+        <v>22502.8450417482</v>
       </c>
       <c r="Z31" s="6" t="n">
-        <f aca="false">M31</f>
-        <v>-85272</v>
+        <f aca="false">SUM(B31:M31)</f>
+        <v>0</v>
       </c>
       <c r="AA31" s="6" t="n">
-        <f aca="false">Y31</f>
-        <v>460662.643699088</v>
+        <f aca="false">SUM(N31:Y31)</f>
+        <v>167893.340866931</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B32" s="7" t="n">
+        <f aca="false">B30-B31</f>
+        <v>-9506</v>
+      </c>
+      <c r="C32" s="7" t="n">
+        <f aca="false">C30-C31</f>
+        <v>-9018</v>
+      </c>
+      <c r="D32" s="7" t="n">
+        <f aca="false">D30-D31</f>
+        <v>-8530</v>
+      </c>
+      <c r="E32" s="7" t="n">
+        <f aca="false">E30-E31</f>
+        <v>-8042</v>
+      </c>
+      <c r="F32" s="7" t="n">
+        <f aca="false">F30-F31</f>
+        <v>-7554</v>
+      </c>
+      <c r="G32" s="7" t="n">
+        <f aca="false">G30-G31</f>
+        <v>-7066</v>
+      </c>
+      <c r="H32" s="7" t="n">
+        <f aca="false">H30-H31</f>
+        <v>-7358</v>
+      </c>
+      <c r="I32" s="7" t="n">
+        <f aca="false">I30-I31</f>
+        <v>-4898</v>
+      </c>
+      <c r="J32" s="7" t="n">
+        <f aca="false">J30-J31</f>
+        <v>-10131</v>
+      </c>
+      <c r="K32" s="7" t="n">
+        <f aca="false">K30-K31</f>
+        <v>-4411</v>
+      </c>
+      <c r="L32" s="7" t="n">
+        <f aca="false">L30-L31</f>
+        <v>3261</v>
+      </c>
+      <c r="M32" s="7" t="n">
+        <f aca="false">M30-M31</f>
+        <v>12417</v>
+      </c>
+      <c r="N32" s="7" t="n">
+        <f aca="false">N30-N31</f>
+        <v>27865</v>
+      </c>
+      <c r="O32" s="7" t="n">
+        <f aca="false">O30-O31</f>
+        <v>34239.88</v>
+      </c>
+      <c r="P32" s="7" t="n">
+        <f aca="false">P30-P31</f>
+        <v>31044.5262</v>
+      </c>
+      <c r="Q32" s="7" t="n">
+        <f aca="false">Q30-Q31</f>
+        <v>36041.448438</v>
+      </c>
+      <c r="R32" s="7" t="n">
+        <f aca="false">R30-R31</f>
+        <v>40988.40145362</v>
+      </c>
+      <c r="S32" s="7" t="n">
+        <f aca="false">S30-S31</f>
+        <v>45885.8849390838</v>
+      </c>
+      <c r="T32" s="7" t="n">
+        <f aca="false">T30-T31</f>
+        <v>50734.393589693</v>
+      </c>
+      <c r="U32" s="7" t="n">
+        <f aca="false">U30-U31</f>
+        <v>55534.417153796</v>
+      </c>
+      <c r="V32" s="7" t="n">
+        <f aca="false">V30-V31</f>
+        <v>53535.6904822581</v>
+      </c>
+      <c r="W32" s="7" t="n">
+        <f aca="false">W30-W31</f>
+        <v>58240.1935774355</v>
+      </c>
+      <c r="X32" s="7" t="n">
+        <f aca="false">X30-X31</f>
+        <v>62897.6516416611</v>
+      </c>
+      <c r="Y32" s="7" t="n">
+        <f aca="false">Y30-Y31</f>
+        <v>67508.5351252445</v>
+      </c>
+      <c r="Z32" s="7" t="n">
+        <f aca="false">SUM(B32:M32)</f>
+        <v>-60836</v>
+      </c>
+      <c r="AA32" s="7" t="n">
+        <f aca="false">SUM(N32:Y32)</f>
+        <v>564516.022600792</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="B33" s="6" t="n">
+        <f aca="false">SUM($B32:B32)</f>
+        <v>-9506</v>
+      </c>
+      <c r="C33" s="6" t="n">
+        <f aca="false">SUM($B32:C32)</f>
+        <v>-18524</v>
+      </c>
+      <c r="D33" s="6" t="n">
+        <f aca="false">SUM($B32:D32)</f>
+        <v>-27054</v>
+      </c>
+      <c r="E33" s="6" t="n">
+        <f aca="false">SUM($B32:E32)</f>
+        <v>-35096</v>
+      </c>
+      <c r="F33" s="6" t="n">
+        <f aca="false">SUM($B32:F32)</f>
+        <v>-42650</v>
+      </c>
+      <c r="G33" s="6" t="n">
+        <f aca="false">SUM($B32:G32)</f>
+        <v>-49716</v>
+      </c>
+      <c r="H33" s="6" t="n">
+        <f aca="false">SUM($B32:H32)</f>
+        <v>-57074</v>
+      </c>
+      <c r="I33" s="6" t="n">
+        <f aca="false">SUM($B32:I32)</f>
+        <v>-61972</v>
+      </c>
+      <c r="J33" s="6" t="n">
+        <f aca="false">SUM($B32:J32)</f>
+        <v>-72103</v>
+      </c>
+      <c r="K33" s="6" t="n">
+        <f aca="false">SUM($B32:K32)</f>
+        <v>-76514</v>
+      </c>
+      <c r="L33" s="6" t="n">
+        <f aca="false">SUM($B32:L32)</f>
+        <v>-73253</v>
+      </c>
+      <c r="M33" s="6" t="n">
+        <f aca="false">SUM($B32:M32)</f>
+        <v>-60836</v>
+      </c>
+      <c r="N33" s="6" t="n">
+        <f aca="false">SUM($B32:N32)</f>
+        <v>-32971</v>
+      </c>
+      <c r="O33" s="6" t="n">
+        <f aca="false">SUM($B32:O32)</f>
+        <v>1268.88</v>
+      </c>
+      <c r="P33" s="6" t="n">
+        <f aca="false">SUM($B32:P32)</f>
+        <v>32313.4062</v>
+      </c>
+      <c r="Q33" s="6" t="n">
+        <f aca="false">SUM($B32:Q32)</f>
+        <v>68354.854638</v>
+      </c>
+      <c r="R33" s="6" t="n">
+        <f aca="false">SUM($B32:R32)</f>
+        <v>109343.25609162</v>
+      </c>
+      <c r="S33" s="6" t="n">
+        <f aca="false">SUM($B32:S32)</f>
+        <v>155229.141030704</v>
+      </c>
+      <c r="T33" s="6" t="n">
+        <f aca="false">SUM($B32:T32)</f>
+        <v>205963.534620397</v>
+      </c>
+      <c r="U33" s="6" t="n">
+        <f aca="false">SUM($B32:U32)</f>
+        <v>261497.951774193</v>
+      </c>
+      <c r="V33" s="6" t="n">
+        <f aca="false">SUM($B32:V32)</f>
+        <v>315033.642256451</v>
+      </c>
+      <c r="W33" s="6" t="n">
+        <f aca="false">SUM($B32:W32)</f>
+        <v>373273.835833886</v>
+      </c>
+      <c r="X33" s="6" t="n">
+        <f aca="false">SUM($B32:X32)</f>
+        <v>436171.487475548</v>
+      </c>
+      <c r="Y33" s="6" t="n">
+        <f aca="false">SUM($B32:Y32)</f>
+        <v>503680.022600792</v>
+      </c>
+      <c r="Z33" s="6" t="n">
+        <f aca="false">M33</f>
+        <v>-60836</v>
+      </c>
+      <c r="AA33" s="6" t="n">
+        <f aca="false">Y33</f>
+        <v>503680.022600792</v>
       </c>
     </row>
   </sheetData>

</xml_diff>